<commit_message>
feat: add versioned self-profile nickname API
</commit_message>
<xml_diff>
--- a/docs/design/foundation/OpenStudy-Foundation-API.xlsx
+++ b/docs/design/foundation/OpenStudy-Foundation-API.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용안내" sheetId="1" r:id="Ra547931ace1e48ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API목록" sheetId="2" r:id="R8afcd95d8c724080"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요청필드" sheetId="3" r:id="R46a6ba25572342f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="응답목록" sheetId="4" r:id="R092241b43e624912"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공통모델" sheetId="5" r:id="R8acef7d72d834646"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="오류·보안" sheetId="6" r:id="Re688c0e864c64516"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="업무규칙" sheetId="7" r:id="R53dd92df3c9042fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="확정정책" sheetId="8" r:id="Rf70a35b2e35d4931"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용안내" sheetId="1" r:id="Rc3e399172a6f4f2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API목록" sheetId="2" r:id="R68c09d83f5574685"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요청필드" sheetId="3" r:id="Re4408afc665e46e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="응답목록" sheetId="4" r:id="R0d2ce9b05502463b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공통모델" sheetId="5" r:id="R268e775d8ed14db0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="오류·보안" sheetId="6" r:id="Ra59a2761e1db4c35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="업무규칙" sheetId="7" r:id="Rbdfb13bedc5744f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="확정정책" sheetId="8" r:id="R5e2132c4cbd74390"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FoundationTable2" displayName="FoundationTable2" ref="A5:G45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FoundationTable2" displayName="FoundationTable2" ref="A5:G46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="operationId"/>
     <x:tableColumn id="2" name="분류"/>
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FoundationTable3" displayName="FoundationTable3" ref="A5:J244" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FoundationTable3" displayName="FoundationTable3" ref="A5:J248" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="operationId"/>
     <x:tableColumn id="2" name="위치"/>
@@ -145,7 +145,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FoundationTable4" displayName="FoundationTable4" ref="A5:F325" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FoundationTable4" displayName="FoundationTable4" ref="A5:F331" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="operationId"/>
     <x:tableColumn id="2" name="HTTP"/>
@@ -159,7 +159,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="FoundationTable5" displayName="FoundationTable5" ref="A5:I289" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="FoundationTable5" displayName="FoundationTable5" ref="A5:I320" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="모델"/>
     <x:tableColumn id="2" name="필드"/>
@@ -190,7 +190,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="FoundationTable7" displayName="FoundationTable7" ref="A5:E45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="FoundationTable7" displayName="FoundationTable7" ref="A5:E46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="operationId"/>
     <x:tableColumn id="2" name="동작"/>
@@ -447,7 +447,7 @@
         <x:v>버전</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>0.1.2-design</x:v>
+        <x:v>0.1.3-profile</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
@@ -455,7 +455,7 @@
         <x:v>범위</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>검토 완료 8개 중분류 / 61개 요구사항 / 40개 API / 57개 모델</x:v>
+        <x:v>검토 완료 8개 중분류 / 61개 요구사항 / 41개 API / 61개 모델</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
@@ -463,7 +463,7 @@
         <x:v>상태</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>구현 전 목표 계약입니다. 기존 로그인과 일부 조회가 있어도 이 엑셀의 전체 기능이 구현되었다는 뜻은 아닙니다.</x:v>
+        <x:v>기반 API 목표 계약과 구현된 M1 닉네임 계약입니다. /me/profile 및 현재 사용자 응답은 Issue #27 구현과 일치하며 나머지 API의 구현 여부는 별도로 확인합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
@@ -495,7 +495,7 @@
         <x:v>배열 / 모델 참조</x:v>
       </x:c>
       <x:c r="B12" s="9" t="str">
-        <x:v>요청필드는 중첩 필드와 oneOf 변형을 펼칩니다. 응답은 상태별 모델을 참조하며, 공통모델에 57개 모델의 모든 직접 필드·참조·조합 규칙을 표시합니다.</x:v>
+        <x:v>요청필드는 중첩 필드와 oneOf 변형을 펼칩니다. 응답은 상태별 모델을 참조하며, 공통모델에 61개 모델의 모든 직접 필드·참조·조합 규칙을 표시합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
@@ -519,7 +519,7 @@
         <x:v>원본</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
-        <x:v>docs/design/foundation/openapi.json | 0.1.2-design | SHA-256 45d6d629cbc2ecfc7efe81ee182b6a0366fe8224a0d7c67d47981119e90c5947</x:v>
+        <x:v>docs/design/foundation/openapi.json | 0.1.3-profile | SHA-256 631395a3dd7bc8a8d08441302d2ff01a8b9e06204ed98312dbde1b433cfced28</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
@@ -527,7 +527,7 @@
         <x:v>관련 문서</x:v>
       </x:c>
       <x:c r="B16" s="9" t="str">
-        <x:v>database.md · api.md · decisions.md · traceability.md · implementation-plan.md</x:v>
+        <x:v>database.md · api.md · profile-api.md · decisions.md · traceability.md · implementation-plan.md</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
@@ -570,7 +570,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>API 목록 | 40 operations</x:v>
+        <x:v>API 목록 | 41 operations</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -1540,10 +1540,33 @@
         <x:v>FR-COM-13, FR-BR-06</x:v>
       </x:c>
     </x:row>
+    <x:row r="46" ht="55" customHeight="1">
+      <x:c r="A46" s="9" t="str">
+        <x:v>updateMyProfile</x:v>
+      </x:c>
+      <x:c r="B46" s="9" t="str">
+        <x:v>me</x:v>
+      </x:c>
+      <x:c r="C46" s="9" t="str">
+        <x:v>PATCH</x:v>
+      </x:c>
+      <x:c r="D46" s="9" t="str">
+        <x:v>/api/me/profile</x:v>
+      </x:c>
+      <x:c r="E46" s="9" t="str">
+        <x:v>본인 닉네임 저장</x:v>
+      </x:c>
+      <x:c r="F46" s="9" t="str">
+        <x:v>WORKSPACE</x:v>
+      </x:c>
+      <x:c r="G46" s="9" t="str">
+        <x:v>FR-SET-01, FR-AUTH-05, FR-AUTH-11, FR-COM-03, FR-COM-06, FR-COM-07, FR-COM-10, FR-COM-14, NFR-OPS-02</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0350154e9e443e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R307c3669e5364fdc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8801,10 +8824,132 @@
       </x:c>
       <x:c r="J244" s="9" t="str"/>
     </x:row>
+    <x:row r="245" ht="28" customHeight="1">
+      <x:c r="A245" s="10" t="str">
+        <x:v>updateMyProfile</x:v>
+      </x:c>
+      <x:c r="B245" s="10" t="str">
+        <x:v>header</x:v>
+      </x:c>
+      <x:c r="C245" s="10" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D245" s="10" t="str">
+        <x:v>X-CSRF-Token</x:v>
+      </x:c>
+      <x:c r="E245" s="10" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="F245" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="G245" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H245" s="10" t="str">
+        <x:v>minLength: 1</x:v>
+      </x:c>
+      <x:c r="I245" s="10" t="str">
+        <x:v>GET /auth/csrf에서 발급. login/logout/accept 후 토큰 재발급.</x:v>
+      </x:c>
+      <x:c r="J245" s="10" t="str"/>
+    </x:row>
+    <x:row r="246" ht="28" customHeight="1">
+      <x:c r="A246" s="9" t="str">
+        <x:v>updateMyProfile</x:v>
+      </x:c>
+      <x:c r="B246" s="9" t="str">
+        <x:v>application/json</x:v>
+      </x:c>
+      <x:c r="C246" s="9" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D246" s="9" t="str">
+        <x:v>(body)</x:v>
+      </x:c>
+      <x:c r="E246" s="9" t="str">
+        <x:v>object</x:v>
+      </x:c>
+      <x:c r="F246" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="G246" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H246" s="9" t="str">
+        <x:v>additionalProperties: false</x:v>
+      </x:c>
+      <x:c r="I246" s="9" t="str"/>
+      <x:c r="J246" s="9" t="str"/>
+    </x:row>
+    <x:row r="247" ht="40" customHeight="1">
+      <x:c r="A247" s="10" t="str">
+        <x:v>updateMyProfile</x:v>
+      </x:c>
+      <x:c r="B247" s="10" t="str">
+        <x:v>application/json</x:v>
+      </x:c>
+      <x:c r="C247" s="10" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D247" s="10" t="str">
+        <x:v>nickname</x:v>
+      </x:c>
+      <x:c r="E247" s="10" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="F247" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="G247" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H247" s="10" t="str">
+        <x:v>minLength: 1
+maxLength: 100</x:v>
+      </x:c>
+      <x:c r="I247" s="10" t="str">
+        <x:v>공백만 있는 값은 422. 원문 길이를 검사한 후 앞뒤 공백을 제거해 저장한다. 기존 VARCHAR(100)에 맞춰 Java UTF-16 길이 100 이하로 검증한다.</x:v>
+      </x:c>
+      <x:c r="J247" s="10" t="str"/>
+    </x:row>
+    <x:row r="248" ht="40" customHeight="1">
+      <x:c r="A248" s="9" t="str">
+        <x:v>updateMyProfile</x:v>
+      </x:c>
+      <x:c r="B248" s="9" t="str">
+        <x:v>application/json</x:v>
+      </x:c>
+      <x:c r="C248" s="9" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D248" s="9" t="str">
+        <x:v>version</x:v>
+      </x:c>
+      <x:c r="E248" s="9" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="F248" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="G248" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H248" s="9" t="str">
+        <x:v>minimum: 1
+maximum: 9007199254740991</x:v>
+      </x:c>
+      <x:c r="I248" s="9" t="str">
+        <x:v>API version=DB version+1. 쓰기 요청에 조회한 값을 전송한다.</x:v>
+      </x:c>
+      <x:c r="J248" s="9" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57da29f37e6948fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfaabd4a105f456f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15399,10 +15544,132 @@
         <x:v>X-Request-ID</x:v>
       </x:c>
     </x:row>
+    <x:row r="326" ht="40" customHeight="1">
+      <x:c r="A326" s="9" t="str">
+        <x:v>updateMyProfile</x:v>
+      </x:c>
+      <x:c r="B326" s="9" t="str">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C326" s="9" t="str">
+        <x:v>application/json</x:v>
+      </x:c>
+      <x:c r="D326" s="9" t="str">
+        <x:v>CurrentUser</x:v>
+      </x:c>
+      <x:c r="E326" s="9" t="str">
+        <x:v>정상 처리. 세부 의미는 operation 설명 참조.</x:v>
+      </x:c>
+      <x:c r="F326" s="9" t="str">
+        <x:v>X-Request-ID
+Cache-Control</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="327" ht="28" customHeight="1">
+      <x:c r="A327" s="10" t="str">
+        <x:v>updateMyProfile</x:v>
+      </x:c>
+      <x:c r="B327" s="10" t="str">
+        <x:v>401</x:v>
+      </x:c>
+      <x:c r="C327" s="10" t="str">
+        <x:v>application/json</x:v>
+      </x:c>
+      <x:c r="D327" s="10" t="str">
+        <x:v>ApiError</x:v>
+      </x:c>
+      <x:c r="E327" s="10" t="str">
+        <x:v>유효한 세션/자격증명 없음</x:v>
+      </x:c>
+      <x:c r="F327" s="10" t="str">
+        <x:v>X-Request-ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="328" ht="28" customHeight="1">
+      <x:c r="A328" s="9" t="str">
+        <x:v>updateMyProfile</x:v>
+      </x:c>
+      <x:c r="B328" s="9" t="str">
+        <x:v>403</x:v>
+      </x:c>
+      <x:c r="C328" s="9" t="str">
+        <x:v>application/json</x:v>
+      </x:c>
+      <x:c r="D328" s="9" t="str">
+        <x:v>ApiError</x:v>
+      </x:c>
+      <x:c r="E328" s="9" t="str">
+        <x:v>지점·역할·행위 권한 부족 또는 CSRF 오류</x:v>
+      </x:c>
+      <x:c r="F328" s="9" t="str">
+        <x:v>X-Request-ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="329" ht="40" customHeight="1">
+      <x:c r="A329" s="10" t="str">
+        <x:v>updateMyProfile</x:v>
+      </x:c>
+      <x:c r="B329" s="10" t="str">
+        <x:v>409</x:v>
+      </x:c>
+      <x:c r="C329" s="10" t="str">
+        <x:v>application/json</x:v>
+      </x:c>
+      <x:c r="D329" s="10" t="str">
+        <x:v>ApiError</x:v>
+      </x:c>
+      <x:c r="E329" s="10" t="str">
+        <x:v>버전·상태·중복·멱등성·최종 관리자 충돌</x:v>
+      </x:c>
+      <x:c r="F329" s="10" t="str">
+        <x:v>X-Request-ID
+Retry-After</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="330" ht="28" customHeight="1">
+      <x:c r="A330" s="9" t="str">
+        <x:v>updateMyProfile</x:v>
+      </x:c>
+      <x:c r="B330" s="9" t="str">
+        <x:v>422</x:v>
+      </x:c>
+      <x:c r="C330" s="9" t="str">
+        <x:v>application/json</x:v>
+      </x:c>
+      <x:c r="D330" s="9" t="str">
+        <x:v>ApiError</x:v>
+      </x:c>
+      <x:c r="E330" s="9" t="str">
+        <x:v>입력 필드·형식·범위 오류</x:v>
+      </x:c>
+      <x:c r="F330" s="9" t="str">
+        <x:v>X-Request-ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="331" ht="28" customHeight="1">
+      <x:c r="A331" s="10" t="str">
+        <x:v>updateMyProfile</x:v>
+      </x:c>
+      <x:c r="B331" s="10" t="str">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C331" s="10" t="str">
+        <x:v>application/json</x:v>
+      </x:c>
+      <x:c r="D331" s="10" t="str">
+        <x:v>ApiError</x:v>
+      </x:c>
+      <x:c r="E331" s="10" t="str">
+        <x:v>내부 오류. 안전한 message와 requestId만 반환</x:v>
+      </x:c>
+      <x:c r="F331" s="10" t="str">
+        <x:v>X-Request-ID</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ba7db33e8894042"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39af0beb1ac5477f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15438,7 +15705,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>모델 사전 | 57 schemas</x:v>
+        <x:v>모델 사전 | 61 schemas</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -17240,7 +17507,7 @@
       <x:c r="H77" s="10" t="str"/>
       <x:c r="I77" s="10" t="str"/>
     </x:row>
-    <x:row r="78" ht="28" customHeight="1">
+    <x:row r="78" ht="55" customHeight="1">
       <x:c r="A78" s="9" t="str">
         <x:v>CurrentUser</x:v>
       </x:c>
@@ -17259,9 +17526,11 @@
       <x:c r="F78" s="9" t="str">
         <x:v>additionalProperties: false</x:v>
       </x:c>
-      <x:c r="G78" s="9" t="str"/>
+      <x:c r="G78" s="9" t="str">
+        <x:v>실제 로그인·GET /me·PATCH /me/profile의 사용자 응답. version은 직원 관리와 같은 계정 version(DB+1)이다. 자격증명과 세션 비밀값을 포함하지 않는다.</x:v>
+      </x:c>
       <x:c r="H78" s="9" t="str">
-        <x:v>Employee</x:v>
+        <x:v>SessionUser</x:v>
       </x:c>
       <x:c r="I78" s="9" t="str"/>
     </x:row>
@@ -17273,7 +17542,7 @@
         <x:v>branches</x:v>
       </x:c>
       <x:c r="C79" s="10" t="str">
-        <x:v>array&lt;Branch&gt;</x:v>
+        <x:v>array&lt;SessionBranch&gt;</x:v>
       </x:c>
       <x:c r="D79" s="10" t="str">
         <x:v>필수</x:v>
@@ -17284,7 +17553,7 @@
       <x:c r="F79" s="10" t="str"/>
       <x:c r="G79" s="10" t="str"/>
       <x:c r="H79" s="10" t="str">
-        <x:v>Branch</x:v>
+        <x:v>SessionBranch</x:v>
       </x:c>
       <x:c r="I79" s="10" t="str"/>
     </x:row>
@@ -22364,10 +22633,753 @@
       <x:c r="H289" s="10" t="str"/>
       <x:c r="I289" s="10" t="str"/>
     </x:row>
+    <x:row r="290" ht="40" customHeight="1">
+      <x:c r="A290" s="9" t="str">
+        <x:v>SessionMembership</x:v>
+      </x:c>
+      <x:c r="B290" s="9" t="str">
+        <x:v>(모델)</x:v>
+      </x:c>
+      <x:c r="C290" s="9" t="str">
+        <x:v>object</x:v>
+      </x:c>
+      <x:c r="D290" s="9" t="str">
+        <x:v>해당 없음</x:v>
+      </x:c>
+      <x:c r="E290" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F290" s="9" t="str">
+        <x:v>additionalProperties: false</x:v>
+      </x:c>
+      <x:c r="G290" s="9" t="str">
+        <x:v>현재 사용자에 반환하는 활성 소속. 직원 관리 Membership의 status/version 편집 계약과 구분한다.</x:v>
+      </x:c>
+      <x:c r="H290" s="9" t="str"/>
+      <x:c r="I290" s="9" t="str"/>
+    </x:row>
+    <x:row r="291" ht="28" customHeight="1">
+      <x:c r="A291" s="10" t="str">
+        <x:v>SessionMembership</x:v>
+      </x:c>
+      <x:c r="B291" s="10" t="str">
+        <x:v>branchId</x:v>
+      </x:c>
+      <x:c r="C291" s="10" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D291" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E291" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F291" s="10" t="str">
+        <x:v>pattern: "^[1-9][0-9]{0,19}$"</x:v>
+      </x:c>
+      <x:c r="G291" s="10" t="str">
+        <x:v>BIGINT UNSIGNED를 표현하는 10진 문자열. 서버는 DB 상한도 검증한다.</x:v>
+      </x:c>
+      <x:c r="H291" s="10" t="str">
+        <x:v>Id</x:v>
+      </x:c>
+      <x:c r="I291" s="10" t="str">
+        <x:v>"1"</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="292" ht="28" customHeight="1">
+      <x:c r="A292" s="9" t="str">
+        <x:v>SessionMembership</x:v>
+      </x:c>
+      <x:c r="B292" s="9" t="str">
+        <x:v>role</x:v>
+      </x:c>
+      <x:c r="C292" s="9" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D292" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E292" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F292" s="9" t="str">
+        <x:v>enum: ["admin","staff"]</x:v>
+      </x:c>
+      <x:c r="G292" s="9" t="str"/>
+      <x:c r="H292" s="9" t="str"/>
+      <x:c r="I292" s="9" t="str"/>
+    </x:row>
+    <x:row r="293" ht="28" customHeight="1">
+      <x:c r="A293" s="10" t="str">
+        <x:v>SessionMembership</x:v>
+      </x:c>
+      <x:c r="B293" s="10" t="str">
+        <x:v>permissions</x:v>
+      </x:c>
+      <x:c r="C293" s="10" t="str">
+        <x:v>array&lt;PermissionCode&gt;</x:v>
+      </x:c>
+      <x:c r="D293" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E293" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F293" s="10" t="str">
+        <x:v>uniqueItems: true</x:v>
+      </x:c>
+      <x:c r="G293" s="10" t="str"/>
+      <x:c r="H293" s="10" t="str">
+        <x:v>Permissions</x:v>
+      </x:c>
+      <x:c r="I293" s="10" t="str"/>
+    </x:row>
+    <x:row r="294" ht="55" customHeight="1">
+      <x:c r="A294" s="9" t="str">
+        <x:v>SessionUser</x:v>
+      </x:c>
+      <x:c r="B294" s="9" t="str">
+        <x:v>(모델)</x:v>
+      </x:c>
+      <x:c r="C294" s="9" t="str">
+        <x:v>object</x:v>
+      </x:c>
+      <x:c r="D294" s="9" t="str">
+        <x:v>해당 없음</x:v>
+      </x:c>
+      <x:c r="E294" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F294" s="9" t="str">
+        <x:v>additionalProperties: false</x:v>
+      </x:c>
+      <x:c r="G294" s="9" t="str">
+        <x:v>실제 로그인·GET /me·PATCH /me/profile의 사용자 응답. version은 직원 관리와 같은 계정 version(DB+1)이다. 자격증명과 세션 비밀값을 포함하지 않는다.</x:v>
+      </x:c>
+      <x:c r="H294" s="9" t="str"/>
+      <x:c r="I294" s="9" t="str"/>
+    </x:row>
+    <x:row r="295" ht="28" customHeight="1">
+      <x:c r="A295" s="10" t="str">
+        <x:v>SessionUser</x:v>
+      </x:c>
+      <x:c r="B295" s="10" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="C295" s="10" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D295" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E295" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F295" s="10" t="str">
+        <x:v>pattern: "^[1-9][0-9]{0,19}$"</x:v>
+      </x:c>
+      <x:c r="G295" s="10" t="str">
+        <x:v>BIGINT UNSIGNED를 표현하는 10진 문자열. 서버는 DB 상한도 검증한다.</x:v>
+      </x:c>
+      <x:c r="H295" s="10" t="str">
+        <x:v>Id</x:v>
+      </x:c>
+      <x:c r="I295" s="10" t="str">
+        <x:v>"1"</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="296" ht="40" customHeight="1">
+      <x:c r="A296" s="9" t="str">
+        <x:v>SessionUser</x:v>
+      </x:c>
+      <x:c r="B296" s="9" t="str">
+        <x:v>version</x:v>
+      </x:c>
+      <x:c r="C296" s="9" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="D296" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E296" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F296" s="9" t="str">
+        <x:v>minimum: 1
+maximum: 9007199254740991</x:v>
+      </x:c>
+      <x:c r="G296" s="9" t="str">
+        <x:v>API version=DB version+1. 쓰기 요청에 조회한 값을 전송한다.</x:v>
+      </x:c>
+      <x:c r="H296" s="9" t="str">
+        <x:v>Version</x:v>
+      </x:c>
+      <x:c r="I296" s="9" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="297" ht="28" customHeight="1">
+      <x:c r="A297" s="10" t="str">
+        <x:v>SessionUser</x:v>
+      </x:c>
+      <x:c r="B297" s="10" t="str">
+        <x:v>createdAt</x:v>
+      </x:c>
+      <x:c r="C297" s="10" t="str">
+        <x:v>string (date-time)</x:v>
+      </x:c>
+      <x:c r="D297" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E297" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F297" s="10" t="str"/>
+      <x:c r="G297" s="10" t="str"/>
+      <x:c r="H297" s="10" t="str"/>
+      <x:c r="I297" s="10" t="str"/>
+    </x:row>
+    <x:row r="298" ht="28" customHeight="1">
+      <x:c r="A298" s="9" t="str">
+        <x:v>SessionUser</x:v>
+      </x:c>
+      <x:c r="B298" s="9" t="str">
+        <x:v>updatedAt</x:v>
+      </x:c>
+      <x:c r="C298" s="9" t="str">
+        <x:v>string (date-time)</x:v>
+      </x:c>
+      <x:c r="D298" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E298" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F298" s="9" t="str"/>
+      <x:c r="G298" s="9" t="str"/>
+      <x:c r="H298" s="9" t="str"/>
+      <x:c r="I298" s="9" t="str"/>
+    </x:row>
+    <x:row r="299" ht="28" customHeight="1">
+      <x:c r="A299" s="10" t="str">
+        <x:v>SessionUser</x:v>
+      </x:c>
+      <x:c r="B299" s="10" t="str">
+        <x:v>branchId</x:v>
+      </x:c>
+      <x:c r="C299" s="10" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D299" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E299" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F299" s="10" t="str"/>
+      <x:c r="G299" s="10" t="str">
+        <x:v>기존 화면 호환값. 인가 근거가 아니며 허용된 첫 지점 ID 또는 all.</x:v>
+      </x:c>
+      <x:c r="H299" s="10" t="str"/>
+      <x:c r="I299" s="10" t="str"/>
+    </x:row>
+    <x:row r="300" ht="28" customHeight="1">
+      <x:c r="A300" s="9" t="str">
+        <x:v>SessionUser</x:v>
+      </x:c>
+      <x:c r="B300" s="9" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="C300" s="9" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D300" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E300" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F300" s="9" t="str"/>
+      <x:c r="G300" s="9" t="str"/>
+      <x:c r="H300" s="9" t="str"/>
+      <x:c r="I300" s="9" t="str"/>
+    </x:row>
+    <x:row r="301" ht="28" customHeight="1">
+      <x:c r="A301" s="10" t="str">
+        <x:v>SessionUser</x:v>
+      </x:c>
+      <x:c r="B301" s="10" t="str">
+        <x:v>email</x:v>
+      </x:c>
+      <x:c r="C301" s="10" t="str">
+        <x:v>string (email)</x:v>
+      </x:c>
+      <x:c r="D301" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E301" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F301" s="10" t="str"/>
+      <x:c r="G301" s="10" t="str"/>
+      <x:c r="H301" s="10" t="str"/>
+      <x:c r="I301" s="10" t="str"/>
+    </x:row>
+    <x:row r="302" ht="28" customHeight="1">
+      <x:c r="A302" s="9" t="str">
+        <x:v>SessionUser</x:v>
+      </x:c>
+      <x:c r="B302" s="9" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="C302" s="9" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D302" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E302" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F302" s="9" t="str">
+        <x:v>enum: ["활성","승인 대기","이용 제한","비활성"]</x:v>
+      </x:c>
+      <x:c r="G302" s="9" t="str"/>
+      <x:c r="H302" s="9" t="str"/>
+      <x:c r="I302" s="9" t="str"/>
+    </x:row>
+    <x:row r="303" ht="28" customHeight="1">
+      <x:c r="A303" s="10" t="str">
+        <x:v>SessionUser</x:v>
+      </x:c>
+      <x:c r="B303" s="10" t="str">
+        <x:v>nickname</x:v>
+      </x:c>
+      <x:c r="C303" s="10" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D303" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E303" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F303" s="10" t="str"/>
+      <x:c r="G303" s="10" t="str"/>
+      <x:c r="H303" s="10" t="str"/>
+      <x:c r="I303" s="10" t="str"/>
+    </x:row>
+    <x:row r="304" ht="28" customHeight="1">
+      <x:c r="A304" s="9" t="str">
+        <x:v>SessionUser</x:v>
+      </x:c>
+      <x:c r="B304" s="9" t="str">
+        <x:v>avatar</x:v>
+      </x:c>
+      <x:c r="C304" s="9" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D304" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E304" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F304" s="9" t="str"/>
+      <x:c r="G304" s="9" t="str"/>
+      <x:c r="H304" s="9" t="str"/>
+      <x:c r="I304" s="9" t="str"/>
+    </x:row>
+    <x:row r="305" ht="28" customHeight="1">
+      <x:c r="A305" s="10" t="str">
+        <x:v>SessionUser</x:v>
+      </x:c>
+      <x:c r="B305" s="10" t="str">
+        <x:v>owner</x:v>
+      </x:c>
+      <x:c r="C305" s="10" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D305" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E305" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F305" s="10" t="str"/>
+      <x:c r="G305" s="10" t="str"/>
+      <x:c r="H305" s="10" t="str"/>
+      <x:c r="I305" s="10" t="str"/>
+    </x:row>
+    <x:row r="306" ht="28" customHeight="1">
+      <x:c r="A306" s="9" t="str">
+        <x:v>SessionUser</x:v>
+      </x:c>
+      <x:c r="B306" s="9" t="str">
+        <x:v>memberships</x:v>
+      </x:c>
+      <x:c r="C306" s="9" t="str">
+        <x:v>array&lt;SessionMembership&gt;</x:v>
+      </x:c>
+      <x:c r="D306" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E306" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F306" s="9" t="str"/>
+      <x:c r="G306" s="9" t="str"/>
+      <x:c r="H306" s="9" t="str">
+        <x:v>SessionMembership</x:v>
+      </x:c>
+      <x:c r="I306" s="9" t="str"/>
+    </x:row>
+    <x:row r="307" ht="28" customHeight="1">
+      <x:c r="A307" s="10" t="str">
+        <x:v>SessionBranch</x:v>
+      </x:c>
+      <x:c r="B307" s="10" t="str">
+        <x:v>(모델)</x:v>
+      </x:c>
+      <x:c r="C307" s="10" t="str">
+        <x:v>object</x:v>
+      </x:c>
+      <x:c r="D307" s="10" t="str">
+        <x:v>해당 없음</x:v>
+      </x:c>
+      <x:c r="E307" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F307" s="10" t="str">
+        <x:v>additionalProperties: false</x:v>
+      </x:c>
+      <x:c r="G307" s="10" t="str"/>
+      <x:c r="H307" s="10" t="str"/>
+      <x:c r="I307" s="10" t="str"/>
+    </x:row>
+    <x:row r="308" ht="28" customHeight="1">
+      <x:c r="A308" s="9" t="str">
+        <x:v>SessionBranch</x:v>
+      </x:c>
+      <x:c r="B308" s="9" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="C308" s="9" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D308" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E308" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F308" s="9" t="str">
+        <x:v>pattern: "^[1-9][0-9]{0,19}$"</x:v>
+      </x:c>
+      <x:c r="G308" s="9" t="str">
+        <x:v>BIGINT UNSIGNED를 표현하는 10진 문자열. 서버는 DB 상한도 검증한다.</x:v>
+      </x:c>
+      <x:c r="H308" s="9" t="str">
+        <x:v>Id</x:v>
+      </x:c>
+      <x:c r="I308" s="9" t="str">
+        <x:v>"1"</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="309" ht="40" customHeight="1">
+      <x:c r="A309" s="10" t="str">
+        <x:v>SessionBranch</x:v>
+      </x:c>
+      <x:c r="B309" s="10" t="str">
+        <x:v>version</x:v>
+      </x:c>
+      <x:c r="C309" s="10" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="D309" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E309" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F309" s="10" t="str">
+        <x:v>minimum: 1
+maximum: 9007199254740991</x:v>
+      </x:c>
+      <x:c r="G309" s="10" t="str">
+        <x:v>API version=DB version+1. 쓰기 요청에 조회한 값을 전송한다.</x:v>
+      </x:c>
+      <x:c r="H309" s="10" t="str">
+        <x:v>Version</x:v>
+      </x:c>
+      <x:c r="I309" s="10" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="310" ht="28" customHeight="1">
+      <x:c r="A310" s="9" t="str">
+        <x:v>SessionBranch</x:v>
+      </x:c>
+      <x:c r="B310" s="9" t="str">
+        <x:v>createdAt</x:v>
+      </x:c>
+      <x:c r="C310" s="9" t="str">
+        <x:v>string (date-time)</x:v>
+      </x:c>
+      <x:c r="D310" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E310" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F310" s="9" t="str"/>
+      <x:c r="G310" s="9" t="str"/>
+      <x:c r="H310" s="9" t="str"/>
+      <x:c r="I310" s="9" t="str"/>
+    </x:row>
+    <x:row r="311" ht="28" customHeight="1">
+      <x:c r="A311" s="10" t="str">
+        <x:v>SessionBranch</x:v>
+      </x:c>
+      <x:c r="B311" s="10" t="str">
+        <x:v>updatedAt</x:v>
+      </x:c>
+      <x:c r="C311" s="10" t="str">
+        <x:v>string (date-time)</x:v>
+      </x:c>
+      <x:c r="D311" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E311" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F311" s="10" t="str"/>
+      <x:c r="G311" s="10" t="str"/>
+      <x:c r="H311" s="10" t="str"/>
+      <x:c r="I311" s="10" t="str"/>
+    </x:row>
+    <x:row r="312" ht="28" customHeight="1">
+      <x:c r="A312" s="9" t="str">
+        <x:v>SessionBranch</x:v>
+      </x:c>
+      <x:c r="B312" s="9" t="str">
+        <x:v>branchId</x:v>
+      </x:c>
+      <x:c r="C312" s="9" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D312" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E312" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F312" s="9" t="str">
+        <x:v>pattern: "^[1-9][0-9]{0,19}$"</x:v>
+      </x:c>
+      <x:c r="G312" s="9" t="str">
+        <x:v>BIGINT UNSIGNED를 표현하는 10진 문자열. 서버는 DB 상한도 검증한다.</x:v>
+      </x:c>
+      <x:c r="H312" s="9" t="str">
+        <x:v>Id</x:v>
+      </x:c>
+      <x:c r="I312" s="9" t="str">
+        <x:v>"1"</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="313" ht="28" customHeight="1">
+      <x:c r="A313" s="10" t="str">
+        <x:v>SessionBranch</x:v>
+      </x:c>
+      <x:c r="B313" s="10" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="C313" s="10" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D313" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E313" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F313" s="10" t="str"/>
+      <x:c r="G313" s="10" t="str"/>
+      <x:c r="H313" s="10" t="str"/>
+      <x:c r="I313" s="10" t="str"/>
+    </x:row>
+    <x:row r="314" ht="28" customHeight="1">
+      <x:c r="A314" s="9" t="str">
+        <x:v>SessionBranch</x:v>
+      </x:c>
+      <x:c r="B314" s="9" t="str">
+        <x:v>address</x:v>
+      </x:c>
+      <x:c r="C314" s="9" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D314" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E314" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F314" s="9" t="str"/>
+      <x:c r="G314" s="9" t="str"/>
+      <x:c r="H314" s="9" t="str"/>
+      <x:c r="I314" s="9" t="str"/>
+    </x:row>
+    <x:row r="315" ht="28" customHeight="1">
+      <x:c r="A315" s="10" t="str">
+        <x:v>SessionBranch</x:v>
+      </x:c>
+      <x:c r="B315" s="10" t="str">
+        <x:v>phone</x:v>
+      </x:c>
+      <x:c r="C315" s="10" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D315" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E315" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F315" s="10" t="str"/>
+      <x:c r="G315" s="10" t="str"/>
+      <x:c r="H315" s="10" t="str"/>
+      <x:c r="I315" s="10" t="str"/>
+    </x:row>
+    <x:row r="316" ht="28" customHeight="1">
+      <x:c r="A316" s="9" t="str">
+        <x:v>SessionBranch</x:v>
+      </x:c>
+      <x:c r="B316" s="9" t="str">
+        <x:v>hours</x:v>
+      </x:c>
+      <x:c r="C316" s="9" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D316" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E316" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F316" s="9" t="str"/>
+      <x:c r="G316" s="9" t="str">
+        <x:v>weeklyHours로 만든 표시용 문자열</x:v>
+      </x:c>
+      <x:c r="H316" s="9" t="str"/>
+      <x:c r="I316" s="9" t="str"/>
+    </x:row>
+    <x:row r="317" ht="28" customHeight="1">
+      <x:c r="A317" s="10" t="str">
+        <x:v>SessionBranch</x:v>
+      </x:c>
+      <x:c r="B317" s="10" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="C317" s="10" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D317" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E317" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F317" s="10" t="str">
+        <x:v>enum: ["운영 중","운영 중지"]</x:v>
+      </x:c>
+      <x:c r="G317" s="10" t="str"/>
+      <x:c r="H317" s="10" t="str"/>
+      <x:c r="I317" s="10" t="str"/>
+    </x:row>
+    <x:row r="318" ht="28" customHeight="1">
+      <x:c r="A318" s="9" t="str">
+        <x:v>ProfileUpdate</x:v>
+      </x:c>
+      <x:c r="B318" s="9" t="str">
+        <x:v>(모델)</x:v>
+      </x:c>
+      <x:c r="C318" s="9" t="str">
+        <x:v>object</x:v>
+      </x:c>
+      <x:c r="D318" s="9" t="str">
+        <x:v>해당 없음</x:v>
+      </x:c>
+      <x:c r="E318" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F318" s="9" t="str">
+        <x:v>additionalProperties: false</x:v>
+      </x:c>
+      <x:c r="G318" s="9" t="str"/>
+      <x:c r="H318" s="9" t="str"/>
+      <x:c r="I318" s="9" t="str"/>
+    </x:row>
+    <x:row r="319" ht="40" customHeight="1">
+      <x:c r="A319" s="10" t="str">
+        <x:v>ProfileUpdate</x:v>
+      </x:c>
+      <x:c r="B319" s="10" t="str">
+        <x:v>nickname</x:v>
+      </x:c>
+      <x:c r="C319" s="10" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D319" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E319" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F319" s="10" t="str">
+        <x:v>minLength: 1
+maxLength: 100</x:v>
+      </x:c>
+      <x:c r="G319" s="10" t="str">
+        <x:v>공백만 있는 값은 422. 원문 길이를 검사한 후 앞뒤 공백을 제거해 저장한다. 기존 VARCHAR(100)에 맞춰 Java UTF-16 길이 100 이하로 검증한다.</x:v>
+      </x:c>
+      <x:c r="H319" s="10" t="str"/>
+      <x:c r="I319" s="10" t="str"/>
+    </x:row>
+    <x:row r="320" ht="40" customHeight="1">
+      <x:c r="A320" s="9" t="str">
+        <x:v>ProfileUpdate</x:v>
+      </x:c>
+      <x:c r="B320" s="9" t="str">
+        <x:v>version</x:v>
+      </x:c>
+      <x:c r="C320" s="9" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="D320" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="E320" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="F320" s="9" t="str">
+        <x:v>minimum: 1
+maximum: 9007199254740991</x:v>
+      </x:c>
+      <x:c r="G320" s="9" t="str">
+        <x:v>API version=DB version+1. 쓰기 요청에 조회한 값을 전송한다.</x:v>
+      </x:c>
+      <x:c r="H320" s="9" t="str">
+        <x:v>Version</x:v>
+      </x:c>
+      <x:c r="I320" s="9" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba97eb9e97b04ea3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbfc6bc9e8104a04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22713,7 +23725,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd70ba2907172474d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83f5bfded26f48b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23433,10 +24445,25 @@
         <x:v>x-event-data-schema: {"$ref":"#/components/schemas/WorkspaceEvent"}</x:v>
       </x:c>
     </x:row>
+    <x:row r="46" ht="85" customHeight="1">
+      <x:c r="A46" s="9" t="str">
+        <x:v>updateMyProfile</x:v>
+      </x:c>
+      <x:c r="B46" s="9" t="str">
+        <x:v>본인 닉네임 저장</x:v>
+      </x:c>
+      <x:c r="C46" s="9" t="str">
+        <x:v>ACTIVE 본인 (OWNER, MANAGER, STAFF)</x:v>
+      </x:c>
+      <x:c r="D46" s="9" t="str">
+        <x:v>확정 M1 계약. ACTIVE WORKSPACE 세션의 본인 ID만 사용하며 쿼리 매개변수와 nickname/version 이외의 본문 필드는 422로 거부한다. 이메일·이름·owner·상태·소속·권한·사진·비밀번호·테마는 변경하지 않는다. 계정 version(DB+1)은 직원·소속 관리자 편집과 공유하며 성공 시 정확히 1 증가한다. 충돌은 VERSION_CONFLICT와 latestVersion, reloadUrl=/api/me를 반환한다. 입력을 보존하고 GET /me로 최신 계정을 확인한 뒤 명시적으로 다시 저장한다. 자동 덮어쓰기는 하지 않는다. 닉네임·updated_by·updated_at·감사 actor/requestId와 전후 snapshot·INVALIDATE outbox를 같은 트랜잭션에 기록한다. SSE 전달 완료를 보장하는 계약은 아니다.</x:v>
+      </x:c>
+      <x:c r="E46" s="9" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29b59339b4654481"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3a796b5020d4653"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23665,7 +24692,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3976aec2f1b407b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9bee160895b4578"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feature: add scoped lookups and committed workspace events
</commit_message>
<xml_diff>
--- a/docs/design/foundation/OpenStudy-Foundation-API.xlsx
+++ b/docs/design/foundation/OpenStudy-Foundation-API.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용안내" sheetId="1" r:id="Rc3e399172a6f4f2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API목록" sheetId="2" r:id="R68c09d83f5574685"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요청필드" sheetId="3" r:id="Re4408afc665e46e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="응답목록" sheetId="4" r:id="R0d2ce9b05502463b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공통모델" sheetId="5" r:id="R268e775d8ed14db0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="오류·보안" sheetId="6" r:id="Ra59a2761e1db4c35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="업무규칙" sheetId="7" r:id="Rbdfb13bedc5744f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="확정정책" sheetId="8" r:id="R5e2132c4cbd74390"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용안내" sheetId="1" r:id="R7a99919d4c7442ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API목록" sheetId="2" r:id="R856f69612e764bd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요청필드" sheetId="3" r:id="R856d42b4ca714e71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="응답목록" sheetId="4" r:id="Rd7085c7615a644c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공통모델" sheetId="5" r:id="Rfe0c141af8764833"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="오류·보안" sheetId="6" r:id="Rcae0771692a04adf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="업무규칙" sheetId="7" r:id="Rabe2f07c1fed48ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="확정정책" sheetId="8" r:id="Rb7e6b09c7a2c40ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FoundationTable2" displayName="FoundationTable2" ref="A5:G46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FoundationTable2" displayName="FoundationTable2" ref="A5:G45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="operationId"/>
     <x:tableColumn id="2" name="분류"/>
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FoundationTable3" displayName="FoundationTable3" ref="A5:J248" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FoundationTable3" displayName="FoundationTable3" ref="A5:J245" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="operationId"/>
     <x:tableColumn id="2" name="위치"/>
@@ -145,7 +145,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FoundationTable4" displayName="FoundationTable4" ref="A5:F331" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FoundationTable4" displayName="FoundationTable4" ref="A5:F323" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="operationId"/>
     <x:tableColumn id="2" name="HTTP"/>
@@ -190,7 +190,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="FoundationTable7" displayName="FoundationTable7" ref="A5:E46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="FoundationTable7" displayName="FoundationTable7" ref="A5:E45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="operationId"/>
     <x:tableColumn id="2" name="동작"/>
@@ -447,7 +447,7 @@
         <x:v>버전</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>0.1.3-profile</x:v>
+        <x:v>0.1.4-workspace</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
@@ -455,15 +455,15 @@
         <x:v>범위</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>검토 완료 8개 중분류 / 61개 요구사항 / 41개 API / 61개 모델</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="28" customHeight="1">
+        <x:v>검토 완료 8개 중분류 / 61개 요구사항 / 40개 API / 61개 모델</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="40" customHeight="1">
       <x:c r="A8" s="9" t="str">
         <x:v>상태</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>기반 API 목표 계약과 구현된 M1 닉네임 계약입니다. /me/profile 및 현재 사용자 응답은 Issue #27 구현과 일치하며 나머지 API의 구현 여부는 별도로 확인합니다.</x:v>
+        <x:v>기반 API 목표 계약과 구현된 M1 닉네임 계약입니다. /me/profile·현재 사용자 응답과 /lookups·단일 인스턴스 /workspace/events는 구현 계약입니다. 나머지 API의 구현 여부는 별도로 확인합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
@@ -519,7 +519,7 @@
         <x:v>원본</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
-        <x:v>docs/design/foundation/openapi.json | 0.1.3-profile | SHA-256 631395a3dd7bc8a8d08441302d2ff01a8b9e06204ed98312dbde1b433cfced28</x:v>
+        <x:v>docs/design/foundation/openapi.json | 0.1.4-workspace | SHA-256 b9d4752fef7c0fa165dbc5ca11fe7427c4236b16130706b2c99d786678474da7</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
@@ -570,7 +570,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>API 목록 | 41 operations</x:v>
+        <x:v>API 목록 | 40 operations</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -1402,171 +1402,148 @@
         <x:v>FR-PROD-03, FR-PROD-06, FR-PROD-09</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="40" customHeight="1">
+    <x:row r="40" ht="28" customHeight="1">
       <x:c r="A40" s="9" t="str">
-        <x:v>deleteProduct</x:v>
+        <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B40" s="9" t="str">
         <x:v>products</x:v>
       </x:c>
       <x:c r="C40" s="9" t="str">
-        <x:v>DELETE</x:v>
+        <x:v>POST</x:v>
       </x:c>
       <x:c r="D40" s="9" t="str">
-        <x:v>/api/products/{id}</x:v>
+        <x:v>/api/products/{id}/status</x:v>
       </x:c>
       <x:c r="E40" s="9" t="str">
-        <x:v>거래 이력 없는 상품 물리 삭제</x:v>
+        <x:v>상품 판매 중지·재개</x:v>
       </x:c>
       <x:c r="F40" s="9" t="str">
         <x:v>WORKSPACE</x:v>
       </x:c>
       <x:c r="G40" s="9" t="str">
-        <x:v>FR-PROD-08, FR-PROD-11, FR-COM-08, FR-COM-10, FR-COM-14</x:v>
+        <x:v>FR-PROD-04, FR-PROD-08</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
       <x:c r="A41" s="10" t="str">
-        <x:v>changeProductStatus</x:v>
+        <x:v>replaceProductBranches</x:v>
       </x:c>
       <x:c r="B41" s="10" t="str">
         <x:v>products</x:v>
       </x:c>
       <x:c r="C41" s="10" t="str">
-        <x:v>POST</x:v>
+        <x:v>PUT</x:v>
       </x:c>
       <x:c r="D41" s="10" t="str">
-        <x:v>/api/products/{id}/status</x:v>
+        <x:v>/api/products/{id}/branches</x:v>
       </x:c>
       <x:c r="E41" s="10" t="str">
-        <x:v>상품 판매 중지·재개</x:v>
+        <x:v>상품 판매 지점 집합 변경</x:v>
       </x:c>
       <x:c r="F41" s="10" t="str">
         <x:v>WORKSPACE</x:v>
       </x:c>
       <x:c r="G41" s="10" t="str">
-        <x:v>FR-PROD-04, FR-PROD-08</x:v>
+        <x:v>FR-PROD-05</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="28" customHeight="1">
       <x:c r="A42" s="9" t="str">
-        <x:v>replaceProductBranches</x:v>
+        <x:v>listProductHistory</x:v>
       </x:c>
       <x:c r="B42" s="9" t="str">
         <x:v>products</x:v>
       </x:c>
       <x:c r="C42" s="9" t="str">
-        <x:v>PUT</x:v>
+        <x:v>GET</x:v>
       </x:c>
       <x:c r="D42" s="9" t="str">
-        <x:v>/api/products/{id}/branches</x:v>
+        <x:v>/api/products/{id}/history</x:v>
       </x:c>
       <x:c r="E42" s="9" t="str">
-        <x:v>상품 판매 지점 집합 변경</x:v>
+        <x:v>상품 가격·구성 변경 이력</x:v>
       </x:c>
       <x:c r="F42" s="9" t="str">
         <x:v>WORKSPACE</x:v>
       </x:c>
       <x:c r="G42" s="9" t="str">
-        <x:v>FR-PROD-05</x:v>
+        <x:v>FR-PROD-07, FR-PROD-11</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="28" customHeight="1">
       <x:c r="A43" s="10" t="str">
-        <x:v>listProductHistory</x:v>
+        <x:v>getLookups</x:v>
       </x:c>
       <x:c r="B43" s="10" t="str">
-        <x:v>products</x:v>
+        <x:v>lookups</x:v>
       </x:c>
       <x:c r="C43" s="10" t="str">
         <x:v>GET</x:v>
       </x:c>
       <x:c r="D43" s="10" t="str">
-        <x:v>/api/products/{id}/history</x:v>
+        <x:v>/api/lookups</x:v>
       </x:c>
       <x:c r="E43" s="10" t="str">
-        <x:v>상품 가격·구성 변경 이력</x:v>
+        <x:v>허용된 기반 선택 데이터</x:v>
       </x:c>
       <x:c r="F43" s="10" t="str">
         <x:v>WORKSPACE</x:v>
       </x:c>
       <x:c r="G43" s="10" t="str">
-        <x:v>FR-PROD-07, FR-PROD-11</x:v>
+        <x:v>FR-BR-06, FR-STAFF-06, FR-COM-02</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="28" customHeight="1">
       <x:c r="A44" s="9" t="str">
-        <x:v>getLookups</x:v>
+        <x:v>subscribeWorkspaceEvents</x:v>
       </x:c>
       <x:c r="B44" s="9" t="str">
-        <x:v>lookups</x:v>
+        <x:v>workspace</x:v>
       </x:c>
       <x:c r="C44" s="9" t="str">
         <x:v>GET</x:v>
       </x:c>
       <x:c r="D44" s="9" t="str">
-        <x:v>/api/lookups</x:v>
+        <x:v>/api/workspace/events</x:v>
       </x:c>
       <x:c r="E44" s="9" t="str">
-        <x:v>허용된 기반 선택 데이터</x:v>
+        <x:v>권한별 화면 갱신 SSE</x:v>
       </x:c>
       <x:c r="F44" s="9" t="str">
         <x:v>WORKSPACE</x:v>
       </x:c>
       <x:c r="G44" s="9" t="str">
-        <x:v>FR-BR-06, FR-STAFF-06, FR-COM-02</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="28" customHeight="1">
+        <x:v>FR-COM-13, FR-BR-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="55" customHeight="1">
       <x:c r="A45" s="10" t="str">
-        <x:v>subscribeWorkspaceEvents</x:v>
+        <x:v>updateMyProfile</x:v>
       </x:c>
       <x:c r="B45" s="10" t="str">
-        <x:v>workspace</x:v>
+        <x:v>me</x:v>
       </x:c>
       <x:c r="C45" s="10" t="str">
-        <x:v>GET</x:v>
+        <x:v>PATCH</x:v>
       </x:c>
       <x:c r="D45" s="10" t="str">
-        <x:v>/api/workspace/events</x:v>
+        <x:v>/api/me/profile</x:v>
       </x:c>
       <x:c r="E45" s="10" t="str">
-        <x:v>권한별 화면 갱신 SSE</x:v>
+        <x:v>본인 닉네임 저장</x:v>
       </x:c>
       <x:c r="F45" s="10" t="str">
         <x:v>WORKSPACE</x:v>
       </x:c>
       <x:c r="G45" s="10" t="str">
-        <x:v>FR-COM-13, FR-BR-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="55" customHeight="1">
-      <x:c r="A46" s="9" t="str">
-        <x:v>updateMyProfile</x:v>
-      </x:c>
-      <x:c r="B46" s="9" t="str">
-        <x:v>me</x:v>
-      </x:c>
-      <x:c r="C46" s="9" t="str">
-        <x:v>PATCH</x:v>
-      </x:c>
-      <x:c r="D46" s="9" t="str">
-        <x:v>/api/me/profile</x:v>
-      </x:c>
-      <x:c r="E46" s="9" t="str">
-        <x:v>본인 닉네임 저장</x:v>
-      </x:c>
-      <x:c r="F46" s="9" t="str">
-        <x:v>WORKSPACE</x:v>
-      </x:c>
-      <x:c r="G46" s="9" t="str">
         <x:v>FR-SET-01, FR-AUTH-05, FR-AUTH-11, FR-COM-03, FR-COM-06, FR-COM-07, FR-COM-10, FR-COM-14, NFR-OPS-02</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R307c3669e5364fdc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60cc29c20ffc496d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8058,7 +8035,7 @@
     </x:row>
     <x:row r="220" ht="28" customHeight="1">
       <x:c r="A220" s="9" t="str">
-        <x:v>deleteProduct</x:v>
+        <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B220" s="9" t="str">
         <x:v>path</x:v>
@@ -8090,7 +8067,7 @@
     </x:row>
     <x:row r="221" ht="40" customHeight="1">
       <x:c r="A221" s="10" t="str">
-        <x:v>deleteProduct</x:v>
+        <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B221" s="10" t="str">
         <x:v>query</x:v>
@@ -8121,7 +8098,7 @@
     </x:row>
     <x:row r="222" ht="28" customHeight="1">
       <x:c r="A222" s="9" t="str">
-        <x:v>deleteProduct</x:v>
+        <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B222" s="9" t="str">
         <x:v>header</x:v>
@@ -8149,403 +8126,399 @@
       </x:c>
       <x:c r="J222" s="9" t="str"/>
     </x:row>
-    <x:row r="223" ht="40" customHeight="1">
+    <x:row r="223" ht="28" customHeight="1">
       <x:c r="A223" s="10" t="str">
-        <x:v>deleteProduct</x:v>
+        <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B223" s="10" t="str">
-        <x:v>query</x:v>
+        <x:v>application/json</x:v>
       </x:c>
       <x:c r="C223" s="10" t="str">
         <x:v>기본</x:v>
       </x:c>
       <x:c r="D223" s="10" t="str">
+        <x:v>(body)</x:v>
+      </x:c>
+      <x:c r="E223" s="10" t="str">
+        <x:v>object</x:v>
+      </x:c>
+      <x:c r="F223" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="G223" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H223" s="10" t="str">
+        <x:v>additionalProperties: false</x:v>
+      </x:c>
+      <x:c r="I223" s="10" t="str"/>
+      <x:c r="J223" s="10" t="str"/>
+    </x:row>
+    <x:row r="224" ht="40" customHeight="1">
+      <x:c r="A224" s="9" t="str">
+        <x:v>changeProductStatus</x:v>
+      </x:c>
+      <x:c r="B224" s="9" t="str">
+        <x:v>application/json</x:v>
+      </x:c>
+      <x:c r="C224" s="9" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D224" s="9" t="str">
         <x:v>version</x:v>
       </x:c>
-      <x:c r="E223" s="10" t="str">
+      <x:c r="E224" s="9" t="str">
         <x:v>integer</x:v>
       </x:c>
-      <x:c r="F223" s="10" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="G223" s="10" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H223" s="10" t="str">
+      <x:c r="F224" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="G224" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H224" s="9" t="str">
         <x:v>minimum: 1
 maximum: 9007199254740991</x:v>
       </x:c>
-      <x:c r="I223" s="10" t="str">
-        <x:v>조회한 상품 version. DELETE는 JSON 본문 없이 이 query 값을 사용.
-API version=DB version+1. 쓰기 요청에 조회한 값을 전송한다.</x:v>
-      </x:c>
-      <x:c r="J223" s="10" t="str">
+      <x:c r="I224" s="9" t="str">
+        <x:v>API version=DB version+1. 쓰기 요청에 조회한 값을 전송한다.</x:v>
+      </x:c>
+      <x:c r="J224" s="9" t="str">
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="224" ht="28" customHeight="1">
-      <x:c r="A224" s="9" t="str">
-        <x:v>changeProductStatus</x:v>
-      </x:c>
-      <x:c r="B224" s="9" t="str">
-        <x:v>path</x:v>
-      </x:c>
-      <x:c r="C224" s="9" t="str">
-        <x:v>기본</x:v>
-      </x:c>
-      <x:c r="D224" s="9" t="str">
-        <x:v>id</x:v>
-      </x:c>
-      <x:c r="E224" s="9" t="str">
-        <x:v>string</x:v>
-      </x:c>
-      <x:c r="F224" s="9" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="G224" s="9" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H224" s="9" t="str">
-        <x:v>pattern: "^[1-9][0-9]{0,19}$"</x:v>
-      </x:c>
-      <x:c r="I224" s="9" t="str">
-        <x:v>BIGINT UNSIGNED를 표현하는 10진 문자열. 서버는 DB 상한도 검증한다.</x:v>
-      </x:c>
-      <x:c r="J224" s="9" t="str">
-        <x:v>"1"</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="225" ht="40" customHeight="1">
+    <x:row r="225" ht="28" customHeight="1">
       <x:c r="A225" s="10" t="str">
         <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B225" s="10" t="str">
-        <x:v>query</x:v>
+        <x:v>application/json</x:v>
       </x:c>
       <x:c r="C225" s="10" t="str">
         <x:v>기본</x:v>
       </x:c>
       <x:c r="D225" s="10" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="E225" s="10" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="F225" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="G225" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H225" s="10" t="str">
+        <x:v>enum: ["판매 중","판매 중지"]</x:v>
+      </x:c>
+      <x:c r="I225" s="10" t="str"/>
+      <x:c r="J225" s="10" t="str"/>
+    </x:row>
+    <x:row r="226" ht="28" customHeight="1">
+      <x:c r="A226" s="9" t="str">
+        <x:v>replaceProductBranches</x:v>
+      </x:c>
+      <x:c r="B226" s="9" t="str">
+        <x:v>path</x:v>
+      </x:c>
+      <x:c r="C226" s="9" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D226" s="9" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="E226" s="9" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="F226" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="G226" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H226" s="9" t="str">
+        <x:v>pattern: "^[1-9][0-9]{0,19}$"</x:v>
+      </x:c>
+      <x:c r="I226" s="9" t="str">
+        <x:v>BIGINT UNSIGNED를 표현하는 10진 문자열. 서버는 DB 상한도 검증한다.</x:v>
+      </x:c>
+      <x:c r="J226" s="9" t="str">
+        <x:v>"1"</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227" ht="40" customHeight="1">
+      <x:c r="A227" s="10" t="str">
+        <x:v>replaceProductBranches</x:v>
+      </x:c>
+      <x:c r="B227" s="10" t="str">
+        <x:v>query</x:v>
+      </x:c>
+      <x:c r="C227" s="10" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D227" s="10" t="str">
         <x:v>scope</x:v>
       </x:c>
-      <x:c r="E225" s="10" t="str">
-        <x:v>string</x:v>
-      </x:c>
-      <x:c r="F225" s="10" t="str">
+      <x:c r="E227" s="10" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="F227" s="10" t="str">
         <x:v>선택</x:v>
       </x:c>
-      <x:c r="G225" s="10" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H225" s="10" t="str">
+      <x:c r="G227" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H227" s="10" t="str">
         <x:v>pattern: "^(all|[1-9][0-9]{0,19})$"
 default: "all"</x:v>
       </x:c>
-      <x:c r="I225" s="10" t="str">
+      <x:c r="I227" s="10" t="str">
         <x:v>all은 허용 지점의 합집합. path/body의 구체적 지점과 교차 검사. 접근 불가 ID는 403.</x:v>
       </x:c>
-      <x:c r="J225" s="10" t="str"/>
-    </x:row>
-    <x:row r="226" ht="28" customHeight="1">
-      <x:c r="A226" s="9" t="str">
-        <x:v>changeProductStatus</x:v>
-      </x:c>
-      <x:c r="B226" s="9" t="str">
+      <x:c r="J227" s="10" t="str"/>
+    </x:row>
+    <x:row r="228" ht="28" customHeight="1">
+      <x:c r="A228" s="9" t="str">
+        <x:v>replaceProductBranches</x:v>
+      </x:c>
+      <x:c r="B228" s="9" t="str">
         <x:v>header</x:v>
-      </x:c>
-      <x:c r="C226" s="9" t="str">
-        <x:v>기본</x:v>
-      </x:c>
-      <x:c r="D226" s="9" t="str">
-        <x:v>X-CSRF-Token</x:v>
-      </x:c>
-      <x:c r="E226" s="9" t="str">
-        <x:v>string</x:v>
-      </x:c>
-      <x:c r="F226" s="9" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="G226" s="9" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H226" s="9" t="str">
-        <x:v>minLength: 1</x:v>
-      </x:c>
-      <x:c r="I226" s="9" t="str">
-        <x:v>GET /auth/csrf에서 발급. login/logout/accept 후 토큰 재발급.</x:v>
-      </x:c>
-      <x:c r="J226" s="9" t="str"/>
-    </x:row>
-    <x:row r="227" ht="28" customHeight="1">
-      <x:c r="A227" s="10" t="str">
-        <x:v>changeProductStatus</x:v>
-      </x:c>
-      <x:c r="B227" s="10" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="C227" s="10" t="str">
-        <x:v>기본</x:v>
-      </x:c>
-      <x:c r="D227" s="10" t="str">
-        <x:v>(body)</x:v>
-      </x:c>
-      <x:c r="E227" s="10" t="str">
-        <x:v>object</x:v>
-      </x:c>
-      <x:c r="F227" s="10" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="G227" s="10" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H227" s="10" t="str">
-        <x:v>additionalProperties: false</x:v>
-      </x:c>
-      <x:c r="I227" s="10" t="str"/>
-      <x:c r="J227" s="10" t="str"/>
-    </x:row>
-    <x:row r="228" ht="40" customHeight="1">
-      <x:c r="A228" s="9" t="str">
-        <x:v>changeProductStatus</x:v>
-      </x:c>
-      <x:c r="B228" s="9" t="str">
-        <x:v>application/json</x:v>
       </x:c>
       <x:c r="C228" s="9" t="str">
         <x:v>기본</x:v>
       </x:c>
       <x:c r="D228" s="9" t="str">
+        <x:v>X-CSRF-Token</x:v>
+      </x:c>
+      <x:c r="E228" s="9" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="F228" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="G228" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H228" s="9" t="str">
+        <x:v>minLength: 1</x:v>
+      </x:c>
+      <x:c r="I228" s="9" t="str">
+        <x:v>GET /auth/csrf에서 발급. login/logout/accept 후 토큰 재발급.</x:v>
+      </x:c>
+      <x:c r="J228" s="9" t="str"/>
+    </x:row>
+    <x:row r="229" ht="28" customHeight="1">
+      <x:c r="A229" s="10" t="str">
+        <x:v>replaceProductBranches</x:v>
+      </x:c>
+      <x:c r="B229" s="10" t="str">
+        <x:v>application/json</x:v>
+      </x:c>
+      <x:c r="C229" s="10" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D229" s="10" t="str">
+        <x:v>(body)</x:v>
+      </x:c>
+      <x:c r="E229" s="10" t="str">
+        <x:v>object</x:v>
+      </x:c>
+      <x:c r="F229" s="10" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="G229" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H229" s="10" t="str">
+        <x:v>additionalProperties: false</x:v>
+      </x:c>
+      <x:c r="I229" s="10" t="str"/>
+      <x:c r="J229" s="10" t="str"/>
+    </x:row>
+    <x:row r="230" ht="40" customHeight="1">
+      <x:c r="A230" s="9" t="str">
+        <x:v>replaceProductBranches</x:v>
+      </x:c>
+      <x:c r="B230" s="9" t="str">
+        <x:v>application/json</x:v>
+      </x:c>
+      <x:c r="C230" s="9" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D230" s="9" t="str">
         <x:v>version</x:v>
       </x:c>
-      <x:c r="E228" s="9" t="str">
+      <x:c r="E230" s="9" t="str">
         <x:v>integer</x:v>
       </x:c>
-      <x:c r="F228" s="9" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="G228" s="9" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H228" s="9" t="str">
+      <x:c r="F230" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="G230" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H230" s="9" t="str">
         <x:v>minimum: 1
 maximum: 9007199254740991</x:v>
       </x:c>
-      <x:c r="I228" s="9" t="str">
+      <x:c r="I230" s="9" t="str">
         <x:v>API version=DB version+1. 쓰기 요청에 조회한 값을 전송한다.</x:v>
       </x:c>
-      <x:c r="J228" s="9" t="str">
+      <x:c r="J230" s="9" t="str">
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="229" ht="28" customHeight="1">
-      <x:c r="A229" s="10" t="str">
-        <x:v>changeProductStatus</x:v>
-      </x:c>
-      <x:c r="B229" s="10" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="C229" s="10" t="str">
-        <x:v>기본</x:v>
-      </x:c>
-      <x:c r="D229" s="10" t="str">
-        <x:v>status</x:v>
-      </x:c>
-      <x:c r="E229" s="10" t="str">
-        <x:v>string</x:v>
-      </x:c>
-      <x:c r="F229" s="10" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="G229" s="10" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H229" s="10" t="str">
-        <x:v>enum: ["판매 중","판매 중지"]</x:v>
-      </x:c>
-      <x:c r="I229" s="10" t="str"/>
-      <x:c r="J229" s="10" t="str"/>
-    </x:row>
-    <x:row r="230" ht="28" customHeight="1">
-      <x:c r="A230" s="9" t="str">
-        <x:v>replaceProductBranches</x:v>
-      </x:c>
-      <x:c r="B230" s="9" t="str">
-        <x:v>path</x:v>
-      </x:c>
-      <x:c r="C230" s="9" t="str">
-        <x:v>기본</x:v>
-      </x:c>
-      <x:c r="D230" s="9" t="str">
-        <x:v>id</x:v>
-      </x:c>
-      <x:c r="E230" s="9" t="str">
-        <x:v>string</x:v>
-      </x:c>
-      <x:c r="F230" s="9" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="G230" s="9" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H230" s="9" t="str">
-        <x:v>pattern: "^[1-9][0-9]{0,19}$"</x:v>
-      </x:c>
-      <x:c r="I230" s="9" t="str">
-        <x:v>BIGINT UNSIGNED를 표현하는 10진 문자열. 서버는 DB 상한도 검증한다.</x:v>
-      </x:c>
-      <x:c r="J230" s="9" t="str">
-        <x:v>"1"</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="231" ht="40" customHeight="1">
+    <x:row r="231" ht="55" customHeight="1">
       <x:c r="A231" s="10" t="str">
         <x:v>replaceProductBranches</x:v>
       </x:c>
       <x:c r="B231" s="10" t="str">
-        <x:v>query</x:v>
+        <x:v>application/json</x:v>
       </x:c>
       <x:c r="C231" s="10" t="str">
         <x:v>기본</x:v>
       </x:c>
       <x:c r="D231" s="10" t="str">
-        <x:v>scope</x:v>
+        <x:v>branchIds</x:v>
       </x:c>
       <x:c r="E231" s="10" t="str">
-        <x:v>string</x:v>
+        <x:v>array&lt;Id&gt;</x:v>
       </x:c>
       <x:c r="F231" s="10" t="str">
-        <x:v>선택</x:v>
+        <x:v>필수</x:v>
       </x:c>
       <x:c r="G231" s="10" t="str">
         <x:v>불가</x:v>
       </x:c>
       <x:c r="H231" s="10" t="str">
-        <x:v>pattern: "^(all|[1-9][0-9]{0,19})$"
-default: "all"</x:v>
-      </x:c>
-      <x:c r="I231" s="10" t="str">
-        <x:v>all은 허용 지점의 합집합. path/body의 구체적 지점과 교차 검사. 접근 불가 ID는 403.</x:v>
-      </x:c>
-      <x:c r="J231" s="10" t="str"/>
-    </x:row>
-    <x:row r="232" ht="28" customHeight="1">
-      <x:c r="A232" s="9" t="str">
-        <x:v>replaceProductBranches</x:v>
-      </x:c>
-      <x:c r="B232" s="9" t="str">
-        <x:v>header</x:v>
-      </x:c>
-      <x:c r="C232" s="9" t="str">
-        <x:v>기본</x:v>
-      </x:c>
-      <x:c r="D232" s="9" t="str">
-        <x:v>X-CSRF-Token</x:v>
-      </x:c>
-      <x:c r="E232" s="9" t="str">
-        <x:v>string</x:v>
-      </x:c>
-      <x:c r="F232" s="9" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="G232" s="9" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H232" s="9" t="str">
-        <x:v>minLength: 1</x:v>
-      </x:c>
-      <x:c r="I232" s="9" t="str">
-        <x:v>GET /auth/csrf에서 발급. login/logout/accept 후 토큰 재발급.</x:v>
-      </x:c>
-      <x:c r="J232" s="9" t="str"/>
-    </x:row>
-    <x:row r="233" ht="28" customHeight="1">
-      <x:c r="A233" s="10" t="str">
-        <x:v>replaceProductBranches</x:v>
-      </x:c>
-      <x:c r="B233" s="10" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="C233" s="10" t="str">
-        <x:v>기본</x:v>
-      </x:c>
-      <x:c r="D233" s="10" t="str">
-        <x:v>(body)</x:v>
-      </x:c>
-      <x:c r="E233" s="10" t="str">
-        <x:v>object</x:v>
-      </x:c>
-      <x:c r="F233" s="10" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="G233" s="10" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H233" s="10" t="str">
-        <x:v>additionalProperties: false</x:v>
-      </x:c>
-      <x:c r="I233" s="10" t="str"/>
-      <x:c r="J233" s="10" t="str"/>
-    </x:row>
-    <x:row r="234" ht="40" customHeight="1">
-      <x:c r="A234" s="9" t="str">
-        <x:v>replaceProductBranches</x:v>
-      </x:c>
-      <x:c r="B234" s="9" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="C234" s="9" t="str">
-        <x:v>기본</x:v>
-      </x:c>
-      <x:c r="D234" s="9" t="str">
-        <x:v>version</x:v>
-      </x:c>
-      <x:c r="E234" s="9" t="str">
-        <x:v>integer</x:v>
-      </x:c>
-      <x:c r="F234" s="9" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="G234" s="9" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H234" s="9" t="str">
-        <x:v>minimum: 1
-maximum: 9007199254740991</x:v>
-      </x:c>
-      <x:c r="I234" s="9" t="str">
-        <x:v>API version=DB version+1. 쓰기 요청에 조회한 값을 전송한다.</x:v>
-      </x:c>
-      <x:c r="J234" s="9" t="str">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="235" ht="55" customHeight="1">
-      <x:c r="A235" s="10" t="str">
-        <x:v>replaceProductBranches</x:v>
-      </x:c>
-      <x:c r="B235" s="10" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="C235" s="10" t="str">
-        <x:v>기본</x:v>
-      </x:c>
-      <x:c r="D235" s="10" t="str">
-        <x:v>branchIds</x:v>
-      </x:c>
-      <x:c r="E235" s="10" t="str">
-        <x:v>array&lt;Id&gt;</x:v>
-      </x:c>
-      <x:c r="F235" s="10" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="G235" s="10" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H235" s="10" t="str">
         <x:v>minItems: 1
 maxItems: 100
 uniqueItems: true</x:v>
       </x:c>
+      <x:c r="I231" s="10" t="str"/>
+      <x:c r="J231" s="10" t="str"/>
+    </x:row>
+    <x:row r="232" ht="28" customHeight="1">
+      <x:c r="A232" s="9" t="str">
+        <x:v>listProductHistory</x:v>
+      </x:c>
+      <x:c r="B232" s="9" t="str">
+        <x:v>path</x:v>
+      </x:c>
+      <x:c r="C232" s="9" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D232" s="9" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="E232" s="9" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="F232" s="9" t="str">
+        <x:v>필수</x:v>
+      </x:c>
+      <x:c r="G232" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H232" s="9" t="str">
+        <x:v>pattern: "^[1-9][0-9]{0,19}$"</x:v>
+      </x:c>
+      <x:c r="I232" s="9" t="str">
+        <x:v>BIGINT UNSIGNED를 표현하는 10진 문자열. 서버는 DB 상한도 검증한다.</x:v>
+      </x:c>
+      <x:c r="J232" s="9" t="str">
+        <x:v>"1"</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="233" ht="40" customHeight="1">
+      <x:c r="A233" s="10" t="str">
+        <x:v>listProductHistory</x:v>
+      </x:c>
+      <x:c r="B233" s="10" t="str">
+        <x:v>query</x:v>
+      </x:c>
+      <x:c r="C233" s="10" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D233" s="10" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="E233" s="10" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="F233" s="10" t="str">
+        <x:v>선택</x:v>
+      </x:c>
+      <x:c r="G233" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H233" s="10" t="str">
+        <x:v>pattern: "^(all|[1-9][0-9]{0,19})$"
+default: "all"</x:v>
+      </x:c>
+      <x:c r="I233" s="10" t="str">
+        <x:v>all은 허용 지점의 합집합. path/body의 구체적 지점과 교차 검사. 접근 불가 ID는 403.</x:v>
+      </x:c>
+      <x:c r="J233" s="10" t="str"/>
+    </x:row>
+    <x:row r="234" ht="55" customHeight="1">
+      <x:c r="A234" s="9" t="str">
+        <x:v>listProductHistory</x:v>
+      </x:c>
+      <x:c r="B234" s="9" t="str">
+        <x:v>query</x:v>
+      </x:c>
+      <x:c r="C234" s="9" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D234" s="9" t="str">
+        <x:v>page</x:v>
+      </x:c>
+      <x:c r="E234" s="9" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="F234" s="9" t="str">
+        <x:v>선택</x:v>
+      </x:c>
+      <x:c r="G234" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H234" s="9" t="str">
+        <x:v>minimum: 1
+maximum: 9007199254740991
+default: 1</x:v>
+      </x:c>
+      <x:c r="I234" s="9" t="str"/>
+      <x:c r="J234" s="9" t="str"/>
+    </x:row>
+    <x:row r="235" ht="55" customHeight="1">
+      <x:c r="A235" s="10" t="str">
+        <x:v>listProductHistory</x:v>
+      </x:c>
+      <x:c r="B235" s="10" t="str">
+        <x:v>query</x:v>
+      </x:c>
+      <x:c r="C235" s="10" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D235" s="10" t="str">
+        <x:v>pageSize</x:v>
+      </x:c>
+      <x:c r="E235" s="10" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="F235" s="10" t="str">
+        <x:v>선택</x:v>
+      </x:c>
+      <x:c r="G235" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H235" s="10" t="str">
+        <x:v>minimum: 1
+maximum: 100
+default: 20</x:v>
+      </x:c>
       <x:c r="I235" s="10" t="str"/>
       <x:c r="J235" s="10" t="str"/>
     </x:row>
@@ -8554,34 +8527,32 @@
         <x:v>listProductHistory</x:v>
       </x:c>
       <x:c r="B236" s="9" t="str">
-        <x:v>path</x:v>
+        <x:v>query</x:v>
       </x:c>
       <x:c r="C236" s="9" t="str">
         <x:v>기본</x:v>
       </x:c>
       <x:c r="D236" s="9" t="str">
-        <x:v>id</x:v>
+        <x:v>q</x:v>
       </x:c>
       <x:c r="E236" s="9" t="str">
         <x:v>string</x:v>
       </x:c>
       <x:c r="F236" s="9" t="str">
-        <x:v>필수</x:v>
+        <x:v>선택</x:v>
       </x:c>
       <x:c r="G236" s="9" t="str">
         <x:v>불가</x:v>
       </x:c>
       <x:c r="H236" s="9" t="str">
-        <x:v>pattern: "^[1-9][0-9]{0,19}$"</x:v>
+        <x:v>maxLength: 100</x:v>
       </x:c>
       <x:c r="I236" s="9" t="str">
-        <x:v>BIGINT UNSIGNED를 표현하는 10진 문자열. 서버는 DB 상한도 검증한다.</x:v>
-      </x:c>
-      <x:c r="J236" s="9" t="str">
-        <x:v>"1"</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="237" ht="40" customHeight="1">
+        <x:v>허용한 name/code/email만 검색. SQL/필드명 직접 입력 아님.</x:v>
+      </x:c>
+      <x:c r="J236" s="9" t="str"/>
+    </x:row>
+    <x:row r="237" ht="28" customHeight="1">
       <x:c r="A237" s="10" t="str">
         <x:v>listProductHistory</x:v>
       </x:c>
@@ -8592,7 +8563,7 @@
         <x:v>기본</x:v>
       </x:c>
       <x:c r="D237" s="10" t="str">
-        <x:v>scope</x:v>
+        <x:v>direction</x:v>
       </x:c>
       <x:c r="E237" s="10" t="str">
         <x:v>string</x:v>
@@ -8604,77 +8575,77 @@
         <x:v>불가</x:v>
       </x:c>
       <x:c r="H237" s="10" t="str">
+        <x:v>enum: ["asc","desc"]</x:v>
+      </x:c>
+      <x:c r="I237" s="10" t="str">
+        <x:v>기본 desc. 최종 id tie-breaker도 같은 방향 적용.</x:v>
+      </x:c>
+      <x:c r="J237" s="10" t="str"/>
+    </x:row>
+    <x:row r="238" ht="28" customHeight="1">
+      <x:c r="A238" s="9" t="str">
+        <x:v>listProductHistory</x:v>
+      </x:c>
+      <x:c r="B238" s="9" t="str">
+        <x:v>query</x:v>
+      </x:c>
+      <x:c r="C238" s="9" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D238" s="9" t="str">
+        <x:v>sort</x:v>
+      </x:c>
+      <x:c r="E238" s="9" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="F238" s="9" t="str">
+        <x:v>선택</x:v>
+      </x:c>
+      <x:c r="G238" s="9" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H238" s="9" t="str">
+        <x:v>enum: ["changedAt"]</x:v>
+      </x:c>
+      <x:c r="I238" s="9" t="str">
+        <x:v>기본 createdAt. 동률은 id로 안정 정렬.</x:v>
+      </x:c>
+      <x:c r="J238" s="9" t="str"/>
+    </x:row>
+    <x:row r="239" ht="40" customHeight="1">
+      <x:c r="A239" s="10" t="str">
+        <x:v>getLookups</x:v>
+      </x:c>
+      <x:c r="B239" s="10" t="str">
+        <x:v>query</x:v>
+      </x:c>
+      <x:c r="C239" s="10" t="str">
+        <x:v>기본</x:v>
+      </x:c>
+      <x:c r="D239" s="10" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="E239" s="10" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="F239" s="10" t="str">
+        <x:v>선택</x:v>
+      </x:c>
+      <x:c r="G239" s="10" t="str">
+        <x:v>불가</x:v>
+      </x:c>
+      <x:c r="H239" s="10" t="str">
         <x:v>pattern: "^(all|[1-9][0-9]{0,19})$"
 default: "all"</x:v>
       </x:c>
-      <x:c r="I237" s="10" t="str">
+      <x:c r="I239" s="10" t="str">
         <x:v>all은 허용 지점의 합집합. path/body의 구체적 지점과 교차 검사. 접근 불가 ID는 403.</x:v>
       </x:c>
-      <x:c r="J237" s="10" t="str"/>
-    </x:row>
-    <x:row r="238" ht="55" customHeight="1">
-      <x:c r="A238" s="9" t="str">
-        <x:v>listProductHistory</x:v>
-      </x:c>
-      <x:c r="B238" s="9" t="str">
-        <x:v>query</x:v>
-      </x:c>
-      <x:c r="C238" s="9" t="str">
-        <x:v>기본</x:v>
-      </x:c>
-      <x:c r="D238" s="9" t="str">
-        <x:v>page</x:v>
-      </x:c>
-      <x:c r="E238" s="9" t="str">
-        <x:v>integer</x:v>
-      </x:c>
-      <x:c r="F238" s="9" t="str">
-        <x:v>선택</x:v>
-      </x:c>
-      <x:c r="G238" s="9" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H238" s="9" t="str">
-        <x:v>minimum: 1
-maximum: 9007199254740991
-default: 1</x:v>
-      </x:c>
-      <x:c r="I238" s="9" t="str"/>
-      <x:c r="J238" s="9" t="str"/>
-    </x:row>
-    <x:row r="239" ht="55" customHeight="1">
-      <x:c r="A239" s="10" t="str">
-        <x:v>listProductHistory</x:v>
-      </x:c>
-      <x:c r="B239" s="10" t="str">
-        <x:v>query</x:v>
-      </x:c>
-      <x:c r="C239" s="10" t="str">
-        <x:v>기본</x:v>
-      </x:c>
-      <x:c r="D239" s="10" t="str">
-        <x:v>pageSize</x:v>
-      </x:c>
-      <x:c r="E239" s="10" t="str">
-        <x:v>integer</x:v>
-      </x:c>
-      <x:c r="F239" s="10" t="str">
-        <x:v>선택</x:v>
-      </x:c>
-      <x:c r="G239" s="10" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H239" s="10" t="str">
-        <x:v>minimum: 1
-maximum: 100
-default: 20</x:v>
-      </x:c>
-      <x:c r="I239" s="10" t="str"/>
       <x:c r="J239" s="10" t="str"/>
     </x:row>
-    <x:row r="240" ht="28" customHeight="1">
+    <x:row r="240" ht="40" customHeight="1">
       <x:c r="A240" s="9" t="str">
-        <x:v>listProductHistory</x:v>
+        <x:v>subscribeWorkspaceEvents</x:v>
       </x:c>
       <x:c r="B240" s="9" t="str">
         <x:v>query</x:v>
@@ -8683,7 +8654,7 @@
         <x:v>기본</x:v>
       </x:c>
       <x:c r="D240" s="9" t="str">
-        <x:v>q</x:v>
+        <x:v>scope</x:v>
       </x:c>
       <x:c r="E240" s="9" t="str">
         <x:v>string</x:v>
@@ -8695,16 +8666,17 @@
         <x:v>불가</x:v>
       </x:c>
       <x:c r="H240" s="9" t="str">
-        <x:v>maxLength: 100</x:v>
+        <x:v>pattern: "^(all|[1-9][0-9]{0,19})$"
+default: "all"</x:v>
       </x:c>
       <x:c r="I240" s="9" t="str">
-        <x:v>허용한 name/code/email만 검색. SQL/필드명 직접 입력 아님.</x:v>
+        <x:v>all은 허용 지점의 합집합. path/body의 구체적 지점과 교차 검사. 접근 불가 ID는 403.</x:v>
       </x:c>
       <x:c r="J240" s="9" t="str"/>
     </x:row>
-    <x:row r="241" ht="28" customHeight="1">
+    <x:row r="241" ht="40" customHeight="1">
       <x:c r="A241" s="10" t="str">
-        <x:v>listProductHistory</x:v>
+        <x:v>subscribeWorkspaceEvents</x:v>
       </x:c>
       <x:c r="B241" s="10" t="str">
         <x:v>query</x:v>
@@ -8713,7 +8685,7 @@
         <x:v>기본</x:v>
       </x:c>
       <x:c r="D241" s="10" t="str">
-        <x:v>direction</x:v>
+        <x:v>cursor</x:v>
       </x:c>
       <x:c r="E241" s="10" t="str">
         <x:v>string</x:v>
@@ -8724,121 +8696,116 @@
       <x:c r="G241" s="10" t="str">
         <x:v>불가</x:v>
       </x:c>
-      <x:c r="H241" s="10" t="str">
-        <x:v>enum: ["asc","desc"]</x:v>
-      </x:c>
+      <x:c r="H241" s="10" t="str"/>
       <x:c r="I241" s="10" t="str">
-        <x:v>기본 desc. 최종 id tie-breaker도 같은 방향 적용.</x:v>
+        <x:v>호환용 연결 힌트. 이 구현은 값을 재생 cursor로 사용하지 않고 항상 resync로 현재 데이터를 다시 조회한다.</x:v>
       </x:c>
       <x:c r="J241" s="10" t="str"/>
     </x:row>
     <x:row r="242" ht="28" customHeight="1">
       <x:c r="A242" s="9" t="str">
-        <x:v>listProductHistory</x:v>
+        <x:v>updateMyProfile</x:v>
       </x:c>
       <x:c r="B242" s="9" t="str">
-        <x:v>query</x:v>
+        <x:v>header</x:v>
       </x:c>
       <x:c r="C242" s="9" t="str">
         <x:v>기본</x:v>
       </x:c>
       <x:c r="D242" s="9" t="str">
-        <x:v>sort</x:v>
+        <x:v>X-CSRF-Token</x:v>
       </x:c>
       <x:c r="E242" s="9" t="str">
         <x:v>string</x:v>
       </x:c>
       <x:c r="F242" s="9" t="str">
-        <x:v>선택</x:v>
+        <x:v>필수</x:v>
       </x:c>
       <x:c r="G242" s="9" t="str">
         <x:v>불가</x:v>
       </x:c>
       <x:c r="H242" s="9" t="str">
-        <x:v>enum: ["changedAt"]</x:v>
+        <x:v>minLength: 1</x:v>
       </x:c>
       <x:c r="I242" s="9" t="str">
-        <x:v>기본 createdAt. 동률은 id로 안정 정렬.</x:v>
+        <x:v>GET /auth/csrf에서 발급. login/logout/accept 후 토큰 재발급.</x:v>
       </x:c>
       <x:c r="J242" s="9" t="str"/>
     </x:row>
-    <x:row r="243" ht="40" customHeight="1">
+    <x:row r="243" ht="28" customHeight="1">
       <x:c r="A243" s="10" t="str">
-        <x:v>getLookups</x:v>
+        <x:v>updateMyProfile</x:v>
       </x:c>
       <x:c r="B243" s="10" t="str">
-        <x:v>query</x:v>
+        <x:v>application/json</x:v>
       </x:c>
       <x:c r="C243" s="10" t="str">
         <x:v>기본</x:v>
       </x:c>
       <x:c r="D243" s="10" t="str">
-        <x:v>scope</x:v>
+        <x:v>(body)</x:v>
       </x:c>
       <x:c r="E243" s="10" t="str">
-        <x:v>string</x:v>
+        <x:v>object</x:v>
       </x:c>
       <x:c r="F243" s="10" t="str">
-        <x:v>선택</x:v>
+        <x:v>필수</x:v>
       </x:c>
       <x:c r="G243" s="10" t="str">
         <x:v>불가</x:v>
       </x:c>
       <x:c r="H243" s="10" t="str">
-        <x:v>pattern: "^(all|[1-9][0-9]{0,19})$"
-default: "all"</x:v>
-      </x:c>
-      <x:c r="I243" s="10" t="str">
-        <x:v>all은 허용 지점의 합집합. path/body의 구체적 지점과 교차 검사. 접근 불가 ID는 403.</x:v>
-      </x:c>
+        <x:v>additionalProperties: false</x:v>
+      </x:c>
+      <x:c r="I243" s="10" t="str"/>
       <x:c r="J243" s="10" t="str"/>
     </x:row>
     <x:row r="244" ht="40" customHeight="1">
       <x:c r="A244" s="9" t="str">
-        <x:v>subscribeWorkspaceEvents</x:v>
+        <x:v>updateMyProfile</x:v>
       </x:c>
       <x:c r="B244" s="9" t="str">
-        <x:v>query</x:v>
+        <x:v>application/json</x:v>
       </x:c>
       <x:c r="C244" s="9" t="str">
         <x:v>기본</x:v>
       </x:c>
       <x:c r="D244" s="9" t="str">
-        <x:v>scope</x:v>
+        <x:v>nickname</x:v>
       </x:c>
       <x:c r="E244" s="9" t="str">
         <x:v>string</x:v>
       </x:c>
       <x:c r="F244" s="9" t="str">
-        <x:v>선택</x:v>
+        <x:v>필수</x:v>
       </x:c>
       <x:c r="G244" s="9" t="str">
         <x:v>불가</x:v>
       </x:c>
       <x:c r="H244" s="9" t="str">
-        <x:v>pattern: "^(all|[1-9][0-9]{0,19})$"
-default: "all"</x:v>
+        <x:v>minLength: 1
+maxLength: 100</x:v>
       </x:c>
       <x:c r="I244" s="9" t="str">
-        <x:v>all은 허용 지점의 합집합. path/body의 구체적 지점과 교차 검사. 접근 불가 ID는 403.</x:v>
+        <x:v>공백만 있는 값은 422. 원문 길이를 검사한 후 앞뒤 공백을 제거해 저장한다. 기존 VARCHAR(100)에 맞춰 Java UTF-16 길이 100 이하로 검증한다.</x:v>
       </x:c>
       <x:c r="J244" s="9" t="str"/>
     </x:row>
-    <x:row r="245" ht="28" customHeight="1">
+    <x:row r="245" ht="40" customHeight="1">
       <x:c r="A245" s="10" t="str">
         <x:v>updateMyProfile</x:v>
       </x:c>
       <x:c r="B245" s="10" t="str">
-        <x:v>header</x:v>
+        <x:v>application/json</x:v>
       </x:c>
       <x:c r="C245" s="10" t="str">
         <x:v>기본</x:v>
       </x:c>
       <x:c r="D245" s="10" t="str">
-        <x:v>X-CSRF-Token</x:v>
+        <x:v>version</x:v>
       </x:c>
       <x:c r="E245" s="10" t="str">
-        <x:v>string</x:v>
+        <x:v>integer</x:v>
       </x:c>
       <x:c r="F245" s="10" t="str">
         <x:v>필수</x:v>
@@ -8847,109 +8814,20 @@
         <x:v>불가</x:v>
       </x:c>
       <x:c r="H245" s="10" t="str">
-        <x:v>minLength: 1</x:v>
-      </x:c>
-      <x:c r="I245" s="10" t="str">
-        <x:v>GET /auth/csrf에서 발급. login/logout/accept 후 토큰 재발급.</x:v>
-      </x:c>
-      <x:c r="J245" s="10" t="str"/>
-    </x:row>
-    <x:row r="246" ht="28" customHeight="1">
-      <x:c r="A246" s="9" t="str">
-        <x:v>updateMyProfile</x:v>
-      </x:c>
-      <x:c r="B246" s="9" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="C246" s="9" t="str">
-        <x:v>기본</x:v>
-      </x:c>
-      <x:c r="D246" s="9" t="str">
-        <x:v>(body)</x:v>
-      </x:c>
-      <x:c r="E246" s="9" t="str">
-        <x:v>object</x:v>
-      </x:c>
-      <x:c r="F246" s="9" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="G246" s="9" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H246" s="9" t="str">
-        <x:v>additionalProperties: false</x:v>
-      </x:c>
-      <x:c r="I246" s="9" t="str"/>
-      <x:c r="J246" s="9" t="str"/>
-    </x:row>
-    <x:row r="247" ht="40" customHeight="1">
-      <x:c r="A247" s="10" t="str">
-        <x:v>updateMyProfile</x:v>
-      </x:c>
-      <x:c r="B247" s="10" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="C247" s="10" t="str">
-        <x:v>기본</x:v>
-      </x:c>
-      <x:c r="D247" s="10" t="str">
-        <x:v>nickname</x:v>
-      </x:c>
-      <x:c r="E247" s="10" t="str">
-        <x:v>string</x:v>
-      </x:c>
-      <x:c r="F247" s="10" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="G247" s="10" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H247" s="10" t="str">
-        <x:v>minLength: 1
-maxLength: 100</x:v>
-      </x:c>
-      <x:c r="I247" s="10" t="str">
-        <x:v>공백만 있는 값은 422. 원문 길이를 검사한 후 앞뒤 공백을 제거해 저장한다. 기존 VARCHAR(100)에 맞춰 Java UTF-16 길이 100 이하로 검증한다.</x:v>
-      </x:c>
-      <x:c r="J247" s="10" t="str"/>
-    </x:row>
-    <x:row r="248" ht="40" customHeight="1">
-      <x:c r="A248" s="9" t="str">
-        <x:v>updateMyProfile</x:v>
-      </x:c>
-      <x:c r="B248" s="9" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="C248" s="9" t="str">
-        <x:v>기본</x:v>
-      </x:c>
-      <x:c r="D248" s="9" t="str">
-        <x:v>version</x:v>
-      </x:c>
-      <x:c r="E248" s="9" t="str">
-        <x:v>integer</x:v>
-      </x:c>
-      <x:c r="F248" s="9" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="G248" s="9" t="str">
-        <x:v>불가</x:v>
-      </x:c>
-      <x:c r="H248" s="9" t="str">
         <x:v>minimum: 1
 maximum: 9007199254740991</x:v>
       </x:c>
-      <x:c r="I248" s="9" t="str">
+      <x:c r="I245" s="10" t="str">
         <x:v>API version=DB version+1. 쓰기 요청에 조회한 값을 전송한다.</x:v>
       </x:c>
-      <x:c r="J248" s="9" t="str">
+      <x:c r="J245" s="10" t="str">
         <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfaabd4a105f456f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25e649c8fe3341da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14567,7 +14445,7 @@
     </x:row>
     <x:row r="278" ht="40" customHeight="1">
       <x:c r="A278" s="9" t="str">
-        <x:v>deleteProduct</x:v>
+        <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B278" s="9" t="str">
         <x:v>200</x:v>
@@ -14576,7 +14454,7 @@
         <x:v>application/json</x:v>
       </x:c>
       <x:c r="D278" s="9" t="str">
-        <x:v>Success</x:v>
+        <x:v>Product</x:v>
       </x:c>
       <x:c r="E278" s="9" t="str">
         <x:v>정상 처리. 세부 의미는 operation 설명 참조.</x:v>
@@ -14588,7 +14466,7 @@
     </x:row>
     <x:row r="279" ht="28" customHeight="1">
       <x:c r="A279" s="10" t="str">
-        <x:v>deleteProduct</x:v>
+        <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B279" s="10" t="str">
         <x:v>401</x:v>
@@ -14608,7 +14486,7 @@
     </x:row>
     <x:row r="280" ht="28" customHeight="1">
       <x:c r="A280" s="9" t="str">
-        <x:v>deleteProduct</x:v>
+        <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B280" s="9" t="str">
         <x:v>403</x:v>
@@ -14628,7 +14506,7 @@
     </x:row>
     <x:row r="281" ht="28" customHeight="1">
       <x:c r="A281" s="10" t="str">
-        <x:v>deleteProduct</x:v>
+        <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B281" s="10" t="str">
         <x:v>404</x:v>
@@ -14648,7 +14526,7 @@
     </x:row>
     <x:row r="282" ht="40" customHeight="1">
       <x:c r="A282" s="9" t="str">
-        <x:v>deleteProduct</x:v>
+        <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B282" s="9" t="str">
         <x:v>409</x:v>
@@ -14669,7 +14547,7 @@
     </x:row>
     <x:row r="283" ht="28" customHeight="1">
       <x:c r="A283" s="10" t="str">
-        <x:v>deleteProduct</x:v>
+        <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B283" s="10" t="str">
         <x:v>422</x:v>
@@ -14689,7 +14567,7 @@
     </x:row>
     <x:row r="284" ht="40" customHeight="1">
       <x:c r="A284" s="9" t="str">
-        <x:v>deleteProduct</x:v>
+        <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B284" s="9" t="str">
         <x:v>429</x:v>
@@ -14710,7 +14588,7 @@
     </x:row>
     <x:row r="285" ht="28" customHeight="1">
       <x:c r="A285" s="10" t="str">
-        <x:v>deleteProduct</x:v>
+        <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B285" s="10" t="str">
         <x:v>500</x:v>
@@ -14730,7 +14608,7 @@
     </x:row>
     <x:row r="286" ht="40" customHeight="1">
       <x:c r="A286" s="9" t="str">
-        <x:v>changeProductStatus</x:v>
+        <x:v>replaceProductBranches</x:v>
       </x:c>
       <x:c r="B286" s="9" t="str">
         <x:v>200</x:v>
@@ -14751,7 +14629,7 @@
     </x:row>
     <x:row r="287" ht="28" customHeight="1">
       <x:c r="A287" s="10" t="str">
-        <x:v>changeProductStatus</x:v>
+        <x:v>replaceProductBranches</x:v>
       </x:c>
       <x:c r="B287" s="10" t="str">
         <x:v>401</x:v>
@@ -14771,7 +14649,7 @@
     </x:row>
     <x:row r="288" ht="28" customHeight="1">
       <x:c r="A288" s="9" t="str">
-        <x:v>changeProductStatus</x:v>
+        <x:v>replaceProductBranches</x:v>
       </x:c>
       <x:c r="B288" s="9" t="str">
         <x:v>403</x:v>
@@ -14791,7 +14669,7 @@
     </x:row>
     <x:row r="289" ht="28" customHeight="1">
       <x:c r="A289" s="10" t="str">
-        <x:v>changeProductStatus</x:v>
+        <x:v>replaceProductBranches</x:v>
       </x:c>
       <x:c r="B289" s="10" t="str">
         <x:v>404</x:v>
@@ -14811,7 +14689,7 @@
     </x:row>
     <x:row r="290" ht="40" customHeight="1">
       <x:c r="A290" s="9" t="str">
-        <x:v>changeProductStatus</x:v>
+        <x:v>replaceProductBranches</x:v>
       </x:c>
       <x:c r="B290" s="9" t="str">
         <x:v>409</x:v>
@@ -14832,7 +14710,7 @@
     </x:row>
     <x:row r="291" ht="28" customHeight="1">
       <x:c r="A291" s="10" t="str">
-        <x:v>changeProductStatus</x:v>
+        <x:v>replaceProductBranches</x:v>
       </x:c>
       <x:c r="B291" s="10" t="str">
         <x:v>422</x:v>
@@ -14852,7 +14730,7 @@
     </x:row>
     <x:row r="292" ht="40" customHeight="1">
       <x:c r="A292" s="9" t="str">
-        <x:v>changeProductStatus</x:v>
+        <x:v>replaceProductBranches</x:v>
       </x:c>
       <x:c r="B292" s="9" t="str">
         <x:v>429</x:v>
@@ -14873,7 +14751,7 @@
     </x:row>
     <x:row r="293" ht="28" customHeight="1">
       <x:c r="A293" s="10" t="str">
-        <x:v>changeProductStatus</x:v>
+        <x:v>replaceProductBranches</x:v>
       </x:c>
       <x:c r="B293" s="10" t="str">
         <x:v>500</x:v>
@@ -14893,7 +14771,7 @@
     </x:row>
     <x:row r="294" ht="40" customHeight="1">
       <x:c r="A294" s="9" t="str">
-        <x:v>replaceProductBranches</x:v>
+        <x:v>listProductHistory</x:v>
       </x:c>
       <x:c r="B294" s="9" t="str">
         <x:v>200</x:v>
@@ -14902,7 +14780,7 @@
         <x:v>application/json</x:v>
       </x:c>
       <x:c r="D294" s="9" t="str">
-        <x:v>Product</x:v>
+        <x:v>ProductRevisionPage</x:v>
       </x:c>
       <x:c r="E294" s="9" t="str">
         <x:v>정상 처리. 세부 의미는 operation 설명 참조.</x:v>
@@ -14914,7 +14792,7 @@
     </x:row>
     <x:row r="295" ht="28" customHeight="1">
       <x:c r="A295" s="10" t="str">
-        <x:v>replaceProductBranches</x:v>
+        <x:v>listProductHistory</x:v>
       </x:c>
       <x:c r="B295" s="10" t="str">
         <x:v>401</x:v>
@@ -14934,7 +14812,7 @@
     </x:row>
     <x:row r="296" ht="28" customHeight="1">
       <x:c r="A296" s="9" t="str">
-        <x:v>replaceProductBranches</x:v>
+        <x:v>listProductHistory</x:v>
       </x:c>
       <x:c r="B296" s="9" t="str">
         <x:v>403</x:v>
@@ -14954,7 +14832,7 @@
     </x:row>
     <x:row r="297" ht="28" customHeight="1">
       <x:c r="A297" s="10" t="str">
-        <x:v>replaceProductBranches</x:v>
+        <x:v>listProductHistory</x:v>
       </x:c>
       <x:c r="B297" s="10" t="str">
         <x:v>404</x:v>
@@ -14974,7 +14852,7 @@
     </x:row>
     <x:row r="298" ht="40" customHeight="1">
       <x:c r="A298" s="9" t="str">
-        <x:v>replaceProductBranches</x:v>
+        <x:v>listProductHistory</x:v>
       </x:c>
       <x:c r="B298" s="9" t="str">
         <x:v>409</x:v>
@@ -14995,7 +14873,7 @@
     </x:row>
     <x:row r="299" ht="28" customHeight="1">
       <x:c r="A299" s="10" t="str">
-        <x:v>replaceProductBranches</x:v>
+        <x:v>listProductHistory</x:v>
       </x:c>
       <x:c r="B299" s="10" t="str">
         <x:v>422</x:v>
@@ -15015,7 +14893,7 @@
     </x:row>
     <x:row r="300" ht="40" customHeight="1">
       <x:c r="A300" s="9" t="str">
-        <x:v>replaceProductBranches</x:v>
+        <x:v>listProductHistory</x:v>
       </x:c>
       <x:c r="B300" s="9" t="str">
         <x:v>429</x:v>
@@ -15036,7 +14914,7 @@
     </x:row>
     <x:row r="301" ht="28" customHeight="1">
       <x:c r="A301" s="10" t="str">
-        <x:v>replaceProductBranches</x:v>
+        <x:v>listProductHistory</x:v>
       </x:c>
       <x:c r="B301" s="10" t="str">
         <x:v>500</x:v>
@@ -15056,7 +14934,7 @@
     </x:row>
     <x:row r="302" ht="40" customHeight="1">
       <x:c r="A302" s="9" t="str">
-        <x:v>listProductHistory</x:v>
+        <x:v>getLookups</x:v>
       </x:c>
       <x:c r="B302" s="9" t="str">
         <x:v>200</x:v>
@@ -15065,7 +14943,7 @@
         <x:v>application/json</x:v>
       </x:c>
       <x:c r="D302" s="9" t="str">
-        <x:v>ProductRevisionPage</x:v>
+        <x:v>Lookups</x:v>
       </x:c>
       <x:c r="E302" s="9" t="str">
         <x:v>정상 처리. 세부 의미는 operation 설명 참조.</x:v>
@@ -15077,7 +14955,7 @@
     </x:row>
     <x:row r="303" ht="28" customHeight="1">
       <x:c r="A303" s="10" t="str">
-        <x:v>listProductHistory</x:v>
+        <x:v>getLookups</x:v>
       </x:c>
       <x:c r="B303" s="10" t="str">
         <x:v>401</x:v>
@@ -15097,7 +14975,7 @@
     </x:row>
     <x:row r="304" ht="28" customHeight="1">
       <x:c r="A304" s="9" t="str">
-        <x:v>listProductHistory</x:v>
+        <x:v>getLookups</x:v>
       </x:c>
       <x:c r="B304" s="9" t="str">
         <x:v>403</x:v>
@@ -15117,7 +14995,7 @@
     </x:row>
     <x:row r="305" ht="28" customHeight="1">
       <x:c r="A305" s="10" t="str">
-        <x:v>listProductHistory</x:v>
+        <x:v>getLookups</x:v>
       </x:c>
       <x:c r="B305" s="10" t="str">
         <x:v>404</x:v>
@@ -15137,7 +15015,7 @@
     </x:row>
     <x:row r="306" ht="40" customHeight="1">
       <x:c r="A306" s="9" t="str">
-        <x:v>listProductHistory</x:v>
+        <x:v>getLookups</x:v>
       </x:c>
       <x:c r="B306" s="9" t="str">
         <x:v>409</x:v>
@@ -15158,7 +15036,7 @@
     </x:row>
     <x:row r="307" ht="28" customHeight="1">
       <x:c r="A307" s="10" t="str">
-        <x:v>listProductHistory</x:v>
+        <x:v>getLookups</x:v>
       </x:c>
       <x:c r="B307" s="10" t="str">
         <x:v>422</x:v>
@@ -15178,7 +15056,7 @@
     </x:row>
     <x:row r="308" ht="40" customHeight="1">
       <x:c r="A308" s="9" t="str">
-        <x:v>listProductHistory</x:v>
+        <x:v>getLookups</x:v>
       </x:c>
       <x:c r="B308" s="9" t="str">
         <x:v>429</x:v>
@@ -15199,7 +15077,7 @@
     </x:row>
     <x:row r="309" ht="28" customHeight="1">
       <x:c r="A309" s="10" t="str">
-        <x:v>listProductHistory</x:v>
+        <x:v>getLookups</x:v>
       </x:c>
       <x:c r="B309" s="10" t="str">
         <x:v>500</x:v>
@@ -15217,30 +15095,31 @@
         <x:v>X-Request-ID</x:v>
       </x:c>
     </x:row>
-    <x:row r="310" ht="40" customHeight="1">
+    <x:row r="310" ht="55" customHeight="1">
       <x:c r="A310" s="9" t="str">
-        <x:v>getLookups</x:v>
+        <x:v>subscribeWorkspaceEvents</x:v>
       </x:c>
       <x:c r="B310" s="9" t="str">
         <x:v>200</x:v>
       </x:c>
       <x:c r="C310" s="9" t="str">
-        <x:v>application/json</x:v>
+        <x:v>text/event-stream</x:v>
       </x:c>
       <x:c r="D310" s="9" t="str">
-        <x:v>Lookups</x:v>
+        <x:v>string</x:v>
       </x:c>
       <x:c r="E310" s="9" t="str">
         <x:v>정상 처리. 세부 의미는 operation 설명 참조.</x:v>
       </x:c>
       <x:c r="F310" s="9" t="str">
         <x:v>X-Request-ID
-Cache-Control</x:v>
+Cache-Control
+X-Accel-Buffering</x:v>
       </x:c>
     </x:row>
     <x:row r="311" ht="28" customHeight="1">
       <x:c r="A311" s="10" t="str">
-        <x:v>getLookups</x:v>
+        <x:v>subscribeWorkspaceEvents</x:v>
       </x:c>
       <x:c r="B311" s="10" t="str">
         <x:v>401</x:v>
@@ -15260,7 +15139,7 @@
     </x:row>
     <x:row r="312" ht="28" customHeight="1">
       <x:c r="A312" s="9" t="str">
-        <x:v>getLookups</x:v>
+        <x:v>subscribeWorkspaceEvents</x:v>
       </x:c>
       <x:c r="B312" s="9" t="str">
         <x:v>403</x:v>
@@ -15280,7 +15159,7 @@
     </x:row>
     <x:row r="313" ht="28" customHeight="1">
       <x:c r="A313" s="10" t="str">
-        <x:v>getLookups</x:v>
+        <x:v>subscribeWorkspaceEvents</x:v>
       </x:c>
       <x:c r="B313" s="10" t="str">
         <x:v>404</x:v>
@@ -15300,7 +15179,7 @@
     </x:row>
     <x:row r="314" ht="40" customHeight="1">
       <x:c r="A314" s="9" t="str">
-        <x:v>getLookups</x:v>
+        <x:v>subscribeWorkspaceEvents</x:v>
       </x:c>
       <x:c r="B314" s="9" t="str">
         <x:v>409</x:v>
@@ -15321,7 +15200,7 @@
     </x:row>
     <x:row r="315" ht="28" customHeight="1">
       <x:c r="A315" s="10" t="str">
-        <x:v>getLookups</x:v>
+        <x:v>subscribeWorkspaceEvents</x:v>
       </x:c>
       <x:c r="B315" s="10" t="str">
         <x:v>422</x:v>
@@ -15341,7 +15220,7 @@
     </x:row>
     <x:row r="316" ht="40" customHeight="1">
       <x:c r="A316" s="9" t="str">
-        <x:v>getLookups</x:v>
+        <x:v>subscribeWorkspaceEvents</x:v>
       </x:c>
       <x:c r="B316" s="9" t="str">
         <x:v>429</x:v>
@@ -15362,7 +15241,7 @@
     </x:row>
     <x:row r="317" ht="28" customHeight="1">
       <x:c r="A317" s="10" t="str">
-        <x:v>getLookups</x:v>
+        <x:v>subscribeWorkspaceEvents</x:v>
       </x:c>
       <x:c r="B317" s="10" t="str">
         <x:v>500</x:v>
@@ -15380,31 +15259,30 @@
         <x:v>X-Request-ID</x:v>
       </x:c>
     </x:row>
-    <x:row r="318" ht="55" customHeight="1">
+    <x:row r="318" ht="40" customHeight="1">
       <x:c r="A318" s="9" t="str">
-        <x:v>subscribeWorkspaceEvents</x:v>
+        <x:v>updateMyProfile</x:v>
       </x:c>
       <x:c r="B318" s="9" t="str">
         <x:v>200</x:v>
       </x:c>
       <x:c r="C318" s="9" t="str">
-        <x:v>text/event-stream</x:v>
+        <x:v>application/json</x:v>
       </x:c>
       <x:c r="D318" s="9" t="str">
-        <x:v>string</x:v>
+        <x:v>CurrentUser</x:v>
       </x:c>
       <x:c r="E318" s="9" t="str">
         <x:v>정상 처리. 세부 의미는 operation 설명 참조.</x:v>
       </x:c>
       <x:c r="F318" s="9" t="str">
         <x:v>X-Request-ID
-Cache-Control
-X-Accel-Buffering</x:v>
+Cache-Control</x:v>
       </x:c>
     </x:row>
     <x:row r="319" ht="28" customHeight="1">
       <x:c r="A319" s="10" t="str">
-        <x:v>subscribeWorkspaceEvents</x:v>
+        <x:v>updateMyProfile</x:v>
       </x:c>
       <x:c r="B319" s="10" t="str">
         <x:v>401</x:v>
@@ -15424,7 +15302,7 @@
     </x:row>
     <x:row r="320" ht="28" customHeight="1">
       <x:c r="A320" s="9" t="str">
-        <x:v>subscribeWorkspaceEvents</x:v>
+        <x:v>updateMyProfile</x:v>
       </x:c>
       <x:c r="B320" s="9" t="str">
         <x:v>403</x:v>
@@ -15442,12 +15320,12 @@
         <x:v>X-Request-ID</x:v>
       </x:c>
     </x:row>
-    <x:row r="321" ht="28" customHeight="1">
+    <x:row r="321" ht="40" customHeight="1">
       <x:c r="A321" s="10" t="str">
-        <x:v>subscribeWorkspaceEvents</x:v>
+        <x:v>updateMyProfile</x:v>
       </x:c>
       <x:c r="B321" s="10" t="str">
-        <x:v>404</x:v>
+        <x:v>409</x:v>
       </x:c>
       <x:c r="C321" s="10" t="str">
         <x:v>application/json</x:v>
@@ -15456,39 +15334,39 @@
         <x:v>ApiError</x:v>
       </x:c>
       <x:c r="E321" s="10" t="str">
-        <x:v>허용된 범위 안의 대상 없음</x:v>
+        <x:v>버전·상태·중복·멱등성·최종 관리자 충돌</x:v>
       </x:c>
       <x:c r="F321" s="10" t="str">
-        <x:v>X-Request-ID</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="322" ht="40" customHeight="1">
-      <x:c r="A322" s="9" t="str">
-        <x:v>subscribeWorkspaceEvents</x:v>
-      </x:c>
-      <x:c r="B322" s="9" t="str">
-        <x:v>409</x:v>
-      </x:c>
-      <x:c r="C322" s="9" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="D322" s="9" t="str">
-        <x:v>ApiError</x:v>
-      </x:c>
-      <x:c r="E322" s="9" t="str">
-        <x:v>버전·상태·중복·멱등성·최종 관리자 충돌</x:v>
-      </x:c>
-      <x:c r="F322" s="9" t="str">
         <x:v>X-Request-ID
 Retry-After</x:v>
       </x:c>
     </x:row>
+    <x:row r="322" ht="28" customHeight="1">
+      <x:c r="A322" s="9" t="str">
+        <x:v>updateMyProfile</x:v>
+      </x:c>
+      <x:c r="B322" s="9" t="str">
+        <x:v>422</x:v>
+      </x:c>
+      <x:c r="C322" s="9" t="str">
+        <x:v>application/json</x:v>
+      </x:c>
+      <x:c r="D322" s="9" t="str">
+        <x:v>ApiError</x:v>
+      </x:c>
+      <x:c r="E322" s="9" t="str">
+        <x:v>입력 필드·형식·범위 오류</x:v>
+      </x:c>
+      <x:c r="F322" s="9" t="str">
+        <x:v>X-Request-ID</x:v>
+      </x:c>
+    </x:row>
     <x:row r="323" ht="28" customHeight="1">
       <x:c r="A323" s="10" t="str">
-        <x:v>subscribeWorkspaceEvents</x:v>
+        <x:v>updateMyProfile</x:v>
       </x:c>
       <x:c r="B323" s="10" t="str">
-        <x:v>422</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="C323" s="10" t="str">
         <x:v>application/json</x:v>
@@ -15497,179 +15375,16 @@
         <x:v>ApiError</x:v>
       </x:c>
       <x:c r="E323" s="10" t="str">
-        <x:v>입력 필드·형식·범위 오류</x:v>
+        <x:v>내부 오류. 안전한 message와 requestId만 반환</x:v>
       </x:c>
       <x:c r="F323" s="10" t="str">
-        <x:v>X-Request-ID</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="324" ht="40" customHeight="1">
-      <x:c r="A324" s="9" t="str">
-        <x:v>subscribeWorkspaceEvents</x:v>
-      </x:c>
-      <x:c r="B324" s="9" t="str">
-        <x:v>429</x:v>
-      </x:c>
-      <x:c r="C324" s="9" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="D324" s="9" t="str">
-        <x:v>ApiError</x:v>
-      </x:c>
-      <x:c r="E324" s="9" t="str">
-        <x:v>요청 제한. Retry-After 참고</x:v>
-      </x:c>
-      <x:c r="F324" s="9" t="str">
-        <x:v>X-Request-ID
-Retry-After</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="325" ht="28" customHeight="1">
-      <x:c r="A325" s="10" t="str">
-        <x:v>subscribeWorkspaceEvents</x:v>
-      </x:c>
-      <x:c r="B325" s="10" t="str">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="C325" s="10" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="D325" s="10" t="str">
-        <x:v>ApiError</x:v>
-      </x:c>
-      <x:c r="E325" s="10" t="str">
-        <x:v>내부 오류. 안전한 message와 requestId만 반환</x:v>
-      </x:c>
-      <x:c r="F325" s="10" t="str">
-        <x:v>X-Request-ID</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="326" ht="40" customHeight="1">
-      <x:c r="A326" s="9" t="str">
-        <x:v>updateMyProfile</x:v>
-      </x:c>
-      <x:c r="B326" s="9" t="str">
-        <x:v>200</x:v>
-      </x:c>
-      <x:c r="C326" s="9" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="D326" s="9" t="str">
-        <x:v>CurrentUser</x:v>
-      </x:c>
-      <x:c r="E326" s="9" t="str">
-        <x:v>정상 처리. 세부 의미는 operation 설명 참조.</x:v>
-      </x:c>
-      <x:c r="F326" s="9" t="str">
-        <x:v>X-Request-ID
-Cache-Control</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="327" ht="28" customHeight="1">
-      <x:c r="A327" s="10" t="str">
-        <x:v>updateMyProfile</x:v>
-      </x:c>
-      <x:c r="B327" s="10" t="str">
-        <x:v>401</x:v>
-      </x:c>
-      <x:c r="C327" s="10" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="D327" s="10" t="str">
-        <x:v>ApiError</x:v>
-      </x:c>
-      <x:c r="E327" s="10" t="str">
-        <x:v>유효한 세션/자격증명 없음</x:v>
-      </x:c>
-      <x:c r="F327" s="10" t="str">
-        <x:v>X-Request-ID</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="328" ht="28" customHeight="1">
-      <x:c r="A328" s="9" t="str">
-        <x:v>updateMyProfile</x:v>
-      </x:c>
-      <x:c r="B328" s="9" t="str">
-        <x:v>403</x:v>
-      </x:c>
-      <x:c r="C328" s="9" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="D328" s="9" t="str">
-        <x:v>ApiError</x:v>
-      </x:c>
-      <x:c r="E328" s="9" t="str">
-        <x:v>지점·역할·행위 권한 부족 또는 CSRF 오류</x:v>
-      </x:c>
-      <x:c r="F328" s="9" t="str">
-        <x:v>X-Request-ID</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="329" ht="40" customHeight="1">
-      <x:c r="A329" s="10" t="str">
-        <x:v>updateMyProfile</x:v>
-      </x:c>
-      <x:c r="B329" s="10" t="str">
-        <x:v>409</x:v>
-      </x:c>
-      <x:c r="C329" s="10" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="D329" s="10" t="str">
-        <x:v>ApiError</x:v>
-      </x:c>
-      <x:c r="E329" s="10" t="str">
-        <x:v>버전·상태·중복·멱등성·최종 관리자 충돌</x:v>
-      </x:c>
-      <x:c r="F329" s="10" t="str">
-        <x:v>X-Request-ID
-Retry-After</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="330" ht="28" customHeight="1">
-      <x:c r="A330" s="9" t="str">
-        <x:v>updateMyProfile</x:v>
-      </x:c>
-      <x:c r="B330" s="9" t="str">
-        <x:v>422</x:v>
-      </x:c>
-      <x:c r="C330" s="9" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="D330" s="9" t="str">
-        <x:v>ApiError</x:v>
-      </x:c>
-      <x:c r="E330" s="9" t="str">
-        <x:v>입력 필드·형식·범위 오류</x:v>
-      </x:c>
-      <x:c r="F330" s="9" t="str">
-        <x:v>X-Request-ID</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="331" ht="28" customHeight="1">
-      <x:c r="A331" s="10" t="str">
-        <x:v>updateMyProfile</x:v>
-      </x:c>
-      <x:c r="B331" s="10" t="str">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="C331" s="10" t="str">
-        <x:v>application/json</x:v>
-      </x:c>
-      <x:c r="D331" s="10" t="str">
-        <x:v>ApiError</x:v>
-      </x:c>
-      <x:c r="E331" s="10" t="str">
-        <x:v>내부 오류. 안전한 message와 requestId만 반환</x:v>
-      </x:c>
-      <x:c r="F331" s="10" t="str">
         <x:v>X-Request-ID</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39af0beb1ac5477f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb97250742e04be2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21559,7 +21274,7 @@
       </x:c>
       <x:c r="I244" s="9" t="str"/>
     </x:row>
-    <x:row r="245" ht="40" customHeight="1">
+    <x:row r="245" ht="70" customHeight="1">
       <x:c r="A245" s="10" t="str">
         <x:v>ProductRevision</x:v>
       </x:c>
@@ -21579,7 +21294,7 @@
         <x:v>additionalProperties: false</x:v>
       </x:c>
       <x:c r="G245" s="10" t="str">
-        <x:v>productId는 원래 상품 ID로 삭제 후에도 유지. 최초 이력 before=null, DELETED 이력 after=null. 모든 관련 지점 관리 권한 확인.</x:v>
+        <x:v>productId는 불변 상품 ID다. 최초 이력 before=null. SRS v1.1에서는 신규 상품 물리 삭제를 제공하지 않는다. 이전 스키마에서 남은 DELETED 이력이 있는 경우에만 과거 이벤트로 해석하고 새로 생성하지 않는다. 관련 지점 관리 권한을 확인한다.</x:v>
       </x:c>
       <x:c r="H245" s="10" t="str"/>
       <x:c r="I245" s="10" t="str"/>
@@ -22499,7 +22214,7 @@
       <x:c r="H283" s="10" t="str"/>
       <x:c r="I283" s="10" t="str"/>
     </x:row>
-    <x:row r="284" ht="40" customHeight="1">
+    <x:row r="284" ht="70" customHeight="1">
       <x:c r="A284" s="9" t="str">
         <x:v>WorkspaceEvent</x:v>
       </x:c>
@@ -22519,7 +22234,7 @@
         <x:v>additionalProperties: false</x:v>
       </x:c>
       <x:c r="G284" s="9" t="str">
-        <x:v>변경 본문·타 지점 목록·개인정보는 보내지 않는다. 수신 후 현재 권한으로 재조회.</x:v>
+        <x:v>변경 본문·타 지점 목록·개인정보는 보내지 않는다. 수신 후 현재 권한으로 재조회. 개인·전역 선택 데이터 알림은 entityId/branchId를 null로 보낸다. 일반 직원이 타 지점/타 직원의 식별자를 받지 않는다. heartbeat는 이 모델이 아닌 comment다.</x:v>
       </x:c>
       <x:c r="H284" s="9" t="str"/>
       <x:c r="I284" s="9" t="str"/>
@@ -23379,7 +23094,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbfc6bc9e8104a04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57e495878e954cf9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23725,7 +23440,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83f5bfded26f48b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf6fb03a82284aca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24345,125 +24060,108 @@
         <x:v>x-policy-decisions: ["Q2","Q6","Q7","Q9"]</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="55" customHeight="1">
+    <x:row r="40" ht="40" customHeight="1">
       <x:c r="A40" s="9" t="str">
-        <x:v>deleteProduct</x:v>
+        <x:v>changeProductStatus</x:v>
       </x:c>
       <x:c r="B40" s="9" t="str">
-        <x:v>거래 이력 없는 상품 물리 삭제</x:v>
+        <x:v>상품 판매 중지·재개</x:v>
       </x:c>
       <x:c r="C40" s="9" t="str">
         <x:v>OWNER 또는 현재 모든 적용 지점 MANAGER + operations:write</x:v>
       </x:c>
       <x:c r="D40" s="9" t="str">
-        <x:v>구매·결제·발급 참조0건일 때만 삭제. 실패·환불 결제도 이력에 포함하며 참조 존재409 PRODUCT_IN_USE. version 필수·불일치409. 현재 판매 지점 연결 제거와 상품 삭제, DELETED revision·감사·이벤트를 한 트랜잭션으로 처리. 변경 이력의 원래 상품 ID와 snapshot은 보존. 삭제 후 일반 상세404, history는 기존 지점 인가로 조회 가능. 반복 삭제404이며 감사 중복 없음.</x:v>
+        <x:v>판매 중지는 기존 구매·발급 이력을 삭제하지 않는다. SRS v1.1 정책상 거래 유무와 무관하게 상품 물리 삭제 API는 없다. 판매 상태 변경은 상품과 기존 구매·발급 이력을 보존한다.</x:v>
       </x:c>
       <x:c r="E40" s="9" t="str">
-        <x:v>x-policy-decisions: ["Q7","Q8"]</x:v>
+        <x:v>x-policy-decisions: ["Q6","Q7"]</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
       <x:c r="A41" s="10" t="str">
-        <x:v>changeProductStatus</x:v>
+        <x:v>replaceProductBranches</x:v>
       </x:c>
       <x:c r="B41" s="10" t="str">
-        <x:v>상품 판매 중지·재개</x:v>
+        <x:v>상품 판매 지점 집합 변경</x:v>
       </x:c>
       <x:c r="C41" s="10" t="str">
-        <x:v>OWNER 또는 현재 모든 적용 지점 MANAGER + operations:write</x:v>
+        <x:v>OWNER 또는 현재·변경후 모든 지점 MANAGER + operations:write</x:v>
       </x:c>
       <x:c r="D41" s="10" t="str">
-        <x:v>판매 중지는 기존 구매·발급 이력을 삭제하지 않는다. 거래 이력 없는 상품만 별도 DELETE 허용(Q8). DB FK로 구매 참조 삭제도 제한.</x:v>
+        <x:v>최소1개 지점. 범위 밖 ID 유입·기존 적용 지점 숨김 제거를403으로 거부. 새 revision으로 과거 적용 범위 보존.</x:v>
       </x:c>
       <x:c r="E41" s="10" t="str">
         <x:v>x-policy-decisions: ["Q6","Q7"]</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="28" customHeight="1">
+    <x:row r="42" ht="55" customHeight="1">
       <x:c r="A42" s="9" t="str">
-        <x:v>replaceProductBranches</x:v>
+        <x:v>listProductHistory</x:v>
       </x:c>
       <x:c r="B42" s="9" t="str">
-        <x:v>상품 판매 지점 집합 변경</x:v>
+        <x:v>상품 가격·구성 변경 이력</x:v>
       </x:c>
       <x:c r="C42" s="9" t="str">
-        <x:v>OWNER 또는 현재·변경후 모든 지점 MANAGER + operations:write</x:v>
+        <x:v>OWNER 또는 현재·이력의 모든 관련 지점 MANAGER + operations:write</x:v>
       </x:c>
       <x:c r="D42" s="9" t="str">
-        <x:v>최소1개 지점. 범위 밖 ID 유입·기존 적용 지점 숨김 제거를403으로 거부. 새 revision으로 과거 적용 범위 보존.</x:v>
+        <x:v>before/after에 당시 분류·조건·지점 snapshot. 상품 변경 이력은 immutable이고 판매 중지·재개 후에도 원래 상품 ID를 유지한다. 일부 지점 사용자에게 타 지점 이력을 노출하지 않으며 이전 snapshot의 권한도 검사한다. 이전 스키마의 DELETED 기록은 과거 데이터 호환 목적으로만 해석한다.</x:v>
       </x:c>
       <x:c r="E42" s="9" t="str">
-        <x:v>x-policy-decisions: ["Q6","Q7"]</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="40" customHeight="1">
+        <x:v>x-policy-decisions: ["Q8"]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="70" customHeight="1">
       <x:c r="A43" s="10" t="str">
-        <x:v>listProductHistory</x:v>
+        <x:v>getLookups</x:v>
       </x:c>
       <x:c r="B43" s="10" t="str">
-        <x:v>상품 가격·구성 변경 이력</x:v>
+        <x:v>허용된 기반 선택 데이터</x:v>
       </x:c>
       <x:c r="C43" s="10" t="str">
-        <x:v>OWNER 또는 현재·이력의 모든 관련 지점 MANAGER + operations:write</x:v>
+        <x:v>활성 계정 + 허용 지점</x:v>
       </x:c>
       <x:c r="D43" s="10" t="str">
-        <x:v>before/after에 당시 분류·조건·지점 snapshot. 이력은 immutable. 일부 지점 사용자에게 타 지점 이력 노출 금지. 삭제된 상품도 원래 상품 ID의 보존 이력으로 조회. 삭제 직전/과거 snapshot의 모든 지점 인가를 검사. DELETED 행의 after=null.</x:v>
-      </x:c>
-      <x:c r="E43" s="10" t="str">
-        <x:v>x-policy-decisions: ["Q8"]</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="40" customHeight="1">
+        <x:v>빈 데이터는 빈 배열. 직원은 허용 지점의 활성 업무 대상 최소 ID/이름만. 초대/PENDING·타지점 정보 미포함. 선택 데이터가 크면 별도 페이지 조회로 전환; 전체 관리 목록의 total/인가를 대신하지 않는다. 현재 구현은 지점·최소 직원·권한 사전·관리 권한별 프리셋이다. 상품/분류는 미구현 업무 데이터를 운영 선택지로 노출하지 않고 빈 배열을 반환한다. 중지 지점은 이력/설정 조회를 위해 status와 함께 반환하며 신규 거래 허용을 뜻하지 않는다.</x:v>
+      </x:c>
+      <x:c r="E43" s="10" t="str"/>
+    </x:row>
+    <x:row r="44" ht="100" customHeight="1">
       <x:c r="A44" s="9" t="str">
-        <x:v>getLookups</x:v>
+        <x:v>subscribeWorkspaceEvents</x:v>
       </x:c>
       <x:c r="B44" s="9" t="str">
-        <x:v>허용된 기반 선택 데이터</x:v>
+        <x:v>권한별 화면 갱신 SSE</x:v>
       </x:c>
       <x:c r="C44" s="9" t="str">
         <x:v>활성 계정 + 허용 지점</x:v>
       </x:c>
       <x:c r="D44" s="9" t="str">
-        <x:v>빈 데이터는 빈 배열. 직원은 허용 지점의 활성 업무 대상 최소 ID/이름만. 초대/PENDING·타지점 정보 미포함. 선택 데이터가 크면 별도 페이지 조회로 전환; 전체 관리 목록의 total/인가를 대신하지 않는다.</x:v>
-      </x:c>
-      <x:c r="E44" s="9" t="str"/>
-    </x:row>
-    <x:row r="45" ht="40" customHeight="1">
+        <x:v>event: invalidate/authorization.changed/resync. data는 WorkspaceEvent JSON. 커밋 후 전달 직전 현재 권한 재검사. heartbeat는 유효 활동 아님. 재연결 즉시 resync 후 현재 화면 재조회. 재생 보장 없음. 권한 회수·만료면 연결 종료. logout 시 클라이언트가 연결/캐시 정리. 기본 500ms마다 현재 JDBC 세션·계정·소속/권한을 재확인한다. 기본 15초 heartbeat는 SSE comment이고 세션 활동/만료를 연장하지 않는다. 권한 변경은 식별자 없는 authorization.changed 후 종료한다. 세션 만료·로그아웃·계정 제한은 payload 없이 종료한다. 모든 연결/재연결에 resync를 보내며 cursor/Last-Event-ID 재생은 제공하지 않는다. 이벤트 ID는 연결별 논리 힌트이며 outbox 전역 순서를 노출하지 않는다. 개인정보 없는 본인 프로필 신호도 resync를 사용한다.</x:v>
+      </x:c>
+      <x:c r="E44" s="9" t="str">
+        <x:v>x-event-data-schema: {"$ref":"#/components/schemas/WorkspaceEvent"}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="85" customHeight="1">
       <x:c r="A45" s="10" t="str">
-        <x:v>subscribeWorkspaceEvents</x:v>
+        <x:v>updateMyProfile</x:v>
       </x:c>
       <x:c r="B45" s="10" t="str">
-        <x:v>권한별 화면 갱신 SSE</x:v>
+        <x:v>본인 닉네임 저장</x:v>
       </x:c>
       <x:c r="C45" s="10" t="str">
-        <x:v>활성 계정 + 허용 지점</x:v>
+        <x:v>ACTIVE 본인 (OWNER, MANAGER, STAFF)</x:v>
       </x:c>
       <x:c r="D45" s="10" t="str">
-        <x:v>event: invalidate/authorization.changed/resync. data는 WorkspaceEvent JSON. 커밋 후 전달 직전 현재 권한 재검사. heartbeat는 유효 활동 아님. 재연결 즉시 resync 후 현재 화면 재조회. 재생 보장 없음. 권한 회수·만료면 연결 종료. logout 시 클라이언트가 연결/캐시 정리.</x:v>
-      </x:c>
-      <x:c r="E45" s="10" t="str">
-        <x:v>x-event-data-schema: {"$ref":"#/components/schemas/WorkspaceEvent"}</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="85" customHeight="1">
-      <x:c r="A46" s="9" t="str">
-        <x:v>updateMyProfile</x:v>
-      </x:c>
-      <x:c r="B46" s="9" t="str">
-        <x:v>본인 닉네임 저장</x:v>
-      </x:c>
-      <x:c r="C46" s="9" t="str">
-        <x:v>ACTIVE 본인 (OWNER, MANAGER, STAFF)</x:v>
-      </x:c>
-      <x:c r="D46" s="9" t="str">
         <x:v>확정 M1 계약. ACTIVE WORKSPACE 세션의 본인 ID만 사용하며 쿼리 매개변수와 nickname/version 이외의 본문 필드는 422로 거부한다. 이메일·이름·owner·상태·소속·권한·사진·비밀번호·테마는 변경하지 않는다. 계정 version(DB+1)은 직원·소속 관리자 편집과 공유하며 성공 시 정확히 1 증가한다. 충돌은 VERSION_CONFLICT와 latestVersion, reloadUrl=/api/me를 반환한다. 입력을 보존하고 GET /me로 최신 계정을 확인한 뒤 명시적으로 다시 저장한다. 자동 덮어쓰기는 하지 않는다. 닉네임·updated_by·updated_at·감사 actor/requestId와 전후 snapshot·INVALIDATE outbox를 같은 트랜잭션에 기록한다. SSE 전달 완료를 보장하는 계약은 아니다.</x:v>
       </x:c>
-      <x:c r="E46" s="9" t="str"/>
+      <x:c r="E45" s="10" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3a796b5020d4653"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90e4f6e515764ee3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24692,7 +24390,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9bee160895b4578"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R523229593083480f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>